<commit_message>
Sensor harness W-1: JST SH 1.0 mm 4P between feedthrough and PCB J3
- Schematic v0.4: J3 = BM04B-SRSS-TB (top entry). Pins 1-2 MK33, 3-4 Pt1000
  2-wire with force/sense split at the J3 pads (68 nets, netlist check 0 errors)
- Parts list: J3 header, SHR-04V-S housing, SSH-003T-P0.2-H contacts, PTFE AWG30 wire
- Mech: J3 and harness in params/CAD/drawings (item 17, notes 5 and 9), PCAP04
  moved directly behind J3, PCB outline and KiCad board zone updated
- Test for harness clearance, J3 height and pin mapping
- Decision log #16; JST SH -25..+85 C rating added to open items

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA2o8uJsqp9Vzsg4b665ev
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500/HMT500_parts_list.xlsx
+++ b/hardware/kicad/HMT500/HMT500_parts_list.xlsx
@@ -262,8 +262,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N55" headerRowCount="1">
-  <autoFilter ref="A1:N55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N58" headerRowCount="1">
+  <autoFilter ref="A1:N58"/>
   <tableColumns count="14">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="분류"/>
@@ -652,15 +652,15 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A7)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A7)</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A7)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A7)</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A7)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A7)</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -679,15 +679,15 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A8)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A8)</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A8)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A8)</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A8)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A8)</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -706,15 +706,15 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A9)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A9)</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A9)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A9)</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A9)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A9)</f>
         <v/>
       </c>
       <c r="E9" s="10">
@@ -733,15 +733,15 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A10)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A10)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A10)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A10)</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A10)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A10)</f>
         <v/>
       </c>
       <c r="E10" s="10">
@@ -760,15 +760,15 @@
         </is>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A11)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A11)</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A11)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A11)</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A11)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A11)</f>
         <v/>
       </c>
       <c r="E11" s="10">
@@ -787,15 +787,15 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A12)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A12)</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A12)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A12)</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A12)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A12)</f>
         <v/>
       </c>
       <c r="E12" s="10">
@@ -810,19 +810,19 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>기구</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A13)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A13)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A13)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A13)</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A13)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A13)</f>
         <v/>
       </c>
       <c r="E13" s="10">
@@ -837,19 +837,19 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="B14" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A14)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A14)</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A14)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A14)</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A14)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A14)</f>
         <v/>
       </c>
       <c r="E14" s="10">
@@ -864,19 +864,19 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="B15" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A15)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A15)</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A15)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A15)</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A15)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A15)</f>
         <v/>
       </c>
       <c r="E15" s="10">
@@ -891,19 +891,19 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>통신</t>
         </is>
       </c>
       <c r="B16" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A16)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A16)</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A16)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A16)</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A16)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A16)</f>
         <v/>
       </c>
       <c r="E16" s="10">
@@ -918,19 +918,19 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>통신</t>
+          <t>기판</t>
         </is>
       </c>
       <c r="B17" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A17)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A17)</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A17)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A17)</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A17)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A17)</f>
         <v/>
       </c>
       <c r="E17" s="10">
@@ -945,19 +945,19 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>기판</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A18)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A18)</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A18)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A18)</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A18)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A18)</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -972,19 +972,19 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A19)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A19)</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A19)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A19)</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A19)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A19)</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -1003,15 +1003,15 @@
         </is>
       </c>
       <c r="B20" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$55,A20)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$58,A20)</f>
         <v/>
       </c>
       <c r="C20" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$55,'부품리스트'!$B$2:$B$55,A20)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A20)</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$55,'부품리스트'!$B$2:$B$55,A20)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A20)</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>기구</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
@@ -2694,34 +2694,34 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>Feedthrough 6P</t>
+          <t>BM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
-          <t>Feedthrough_6P</t>
+          <t>JST_SH_BM04B-SRSS-TB_1x04-1MP_P1.00mm_Vertical</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>HMT500-P-201</t>
+          <t>BM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>유리-금속 피드스루 6핀 (기구 부품, 바디에 용접)</t>
+          <t>SH 1.0 mm 4핀 헤더, 윗면 삽입 SMD (센서 하네스 W-1, 정격 −25~+85 °C)</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="L26" s="20">
         <f>D26*J26</f>
@@ -2731,9 +2731,9 @@
         <f>D26*K26</f>
         <v/>
       </c>
-      <c r="N26" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N26" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="I48" s="17" t="inlineStr">
         <is>
-          <t>24-bit ADC, Pt1000 4선, TSSOP-16</t>
+          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
         </is>
       </c>
       <c r="J48" s="19" t="n">
@@ -4383,12 +4383,12 @@
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>MK 계열 (사내 공급품)</t>
+          <t>MK33-W mini (150138)</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
         <is>
-          <t>정전용량 습도 소자 (캐리어에 실장)</t>
+          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J53" s="19" t="n">
@@ -4440,17 +4440,17 @@
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>Pt1000 박막 Class A</t>
+          <t>MiniSens Pt1000 F0.1</t>
         </is>
       </c>
       <c r="I54" s="17" t="inlineStr">
         <is>
-          <t>온도 소자 (캐리어에 실장)</t>
+          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J54" s="19" t="n">
@@ -4479,12 +4479,12 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>조립</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-1</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
@@ -4502,24 +4502,24 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>SMT 양면 실장</t>
+          <t>SHR-04V-S</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
         <is>
-          <t>1k 기준 조립비</t>
+          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
         </is>
       </c>
       <c r="J55" s="19" t="n">
-        <v>2</v>
+        <v>0.04</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>4</v>
+        <v>0.1</v>
       </c>
       <c r="L55" s="20">
         <f>D55*J55</f>
@@ -4529,24 +4529,210 @@
         <f>D55*K55</f>
         <v/>
       </c>
-      <c r="N55" s="21" t="inlineStr">
+      <c r="N55" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="16" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="H56" s="17" t="inlineStr">
+        <is>
+          <t>SSH-003T-P0.2-H</t>
+        </is>
+      </c>
+      <c r="I56" s="17" t="inlineStr">
+        <is>
+          <t>SH 크림프 단자 AWG 32–28</t>
+        </is>
+      </c>
+      <c r="J56" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K56" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L56" s="20">
+        <f>D56*J56</f>
+        <v/>
+      </c>
+      <c r="M56" s="20">
+        <f>D56*K56</f>
+        <v/>
+      </c>
+      <c r="N56" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="16" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D57" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E57" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G57" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H57" s="17" t="inlineStr">
+        <is>
+          <t>PTFE AWG30 전선</t>
+        </is>
+      </c>
+      <c r="I57" s="17" t="inlineStr">
+        <is>
+          <t>UL1213 계열 200 °C, 4심 × 22 mm + 수축튜브 (피드스루 핀 납땜)</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K57" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L57" s="20">
+        <f>D57*J57</f>
+        <v/>
+      </c>
+      <c r="M57" s="20">
+        <f>D57*K57</f>
+        <v/>
+      </c>
+      <c r="N57" s="21" t="inlineStr">
         <is>
           <t>추정</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="I56" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="16" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>조립</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G58" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H58" s="17" t="inlineStr">
+        <is>
+          <t>SMT 양면 실장</t>
+        </is>
+      </c>
+      <c r="I58" s="17" t="inlineStr">
+        <is>
+          <t>1k 기준 조립비</t>
+        </is>
+      </c>
+      <c r="J58" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L58" s="20">
+        <f>D58*J58</f>
+        <v/>
+      </c>
+      <c r="M58" s="20">
+        <f>D58*K58</f>
+        <v/>
+      </c>
+      <c r="N58" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="I59" s="3" t="inlineStr">
         <is>
           <t>합계 (1대분)</t>
         </is>
       </c>
-      <c r="L56" s="23">
-        <f>SUM(L2:L55)</f>
-        <v/>
-      </c>
-      <c r="M56" s="23">
-        <f>SUM(M2:M55)</f>
+      <c r="L59" s="23">
+        <f>SUM(L2:L58)</f>
+        <v/>
+      </c>
+      <c r="M59" s="23">
+        <f>SUM(M2:M58)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
M12 field harness W-2 with JST GH 8P, epoxy-molded pass-through
- Schematic v0.5: J1 = JST GH 1.25 mm 8P side entry (SM08B-GHS-TB), pin n =
  M12 pin n; J5 chassis spring contact replaces the M12 shell pin (68 nets, 0 errors)
- Mech: J1 at PCB x 52.5-58.5 facing the connector, harness W-2 (PTFE AWG28, 60 mm)
  and plug in CAD/drawings (item 18, note 10); output-zone parts rearranged
- 7 mm pass-through filled with epoxy over its full length after the cable is in
  (item 5, primary barrier)
- Parts list, KiCad board zones, RFQ, docs, decision log #18 and tests updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA2o8uJsqp9Vzsg4b665ev
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500/HMT500_parts_list.xlsx
+++ b/hardware/kicad/HMT500/HMT500_parts_list.xlsx
@@ -262,8 +262,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N58" headerRowCount="1">
-  <autoFilter ref="A1:N58"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N63" headerRowCount="1">
+  <autoFilter ref="A1:N63"/>
   <tableColumns count="14">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="분류"/>
@@ -652,15 +652,15 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A7)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A7)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A7)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -679,15 +679,15 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A8)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A8)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A8)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -706,15 +706,15 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A9)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A9)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A9)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="E9" s="10">
@@ -733,15 +733,15 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A10)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A10)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A10)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="E10" s="10">
@@ -760,15 +760,15 @@
         </is>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A11)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A11)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A11)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="E11" s="10">
@@ -787,15 +787,15 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A12)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A12)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A12)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="E12" s="10">
@@ -814,15 +814,15 @@
         </is>
       </c>
       <c r="B13" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A13)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A13)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A13)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="E13" s="10">
@@ -841,15 +841,15 @@
         </is>
       </c>
       <c r="B14" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A14)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A14)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A14)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="E14" s="10">
@@ -868,15 +868,15 @@
         </is>
       </c>
       <c r="B15" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A15)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A15)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A15)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="E15" s="10">
@@ -895,15 +895,15 @@
         </is>
       </c>
       <c r="B16" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A16)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A16)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A16)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="E16" s="10">
@@ -922,15 +922,15 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A17)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A17)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A17)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="E17" s="10">
@@ -949,15 +949,15 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A18)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A18)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A18)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -976,15 +976,15 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A19)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A19)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A19)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -1003,15 +1003,15 @@
         </is>
       </c>
       <c r="B20" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$58,A20)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A20)</f>
         <v/>
       </c>
       <c r="C20" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$58,'부품리스트'!$B$2:$B$58,A20)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A20)</f>
         <v/>
       </c>
       <c r="D20" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$58,'부품리스트'!$B$2:$B$58,A20)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A20)</f>
         <v/>
       </c>
       <c r="E20" s="10">
@@ -1096,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2570,34 +2570,34 @@
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
-          <t>M Connect 8P male</t>
+          <t>SM08B-GHS-TB</t>
         </is>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
-          <t>M_Connect_8P</t>
+          <t>JST_GH_SM08B-GHS-TB_1x08-1MP_P1.25mm_Horizontal</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
         <is>
-          <t>M Connect</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>TBD (두텍 사용품)</t>
+          <t>SM08B-GHS-TB</t>
         </is>
       </c>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>M12 8핀 수컷 전면 장착형, M16×1.5</t>
+          <t>GH 1.25 mm 8핀 헤더, 옆 삽입(직각) SMD (M12 하네스 W-2, 정격 −25~+85 °C)</t>
         </is>
       </c>
       <c r="J24" s="19" t="n">
-        <v>2</v>
+        <v>0.35</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>10</v>
+        <v>0.8</v>
       </c>
       <c r="L24" s="20">
         <f>D24*J24</f>
@@ -2607,9 +2607,9 @@
         <f>D24*K24</f>
         <v/>
       </c>
-      <c r="N24" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N24" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -2743,12 +2743,12 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="D27" s="18" t="n">
@@ -2756,34 +2756,34 @@
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>CMC 2x1mH 0.3A</t>
+          <t>Chassis contact</t>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>CMC_WE-SL</t>
+          <t>Chassis_Spring_Contact</t>
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>Würth</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>WE-SL2 계열 (품번 확인)</t>
+          <t>SMD 스프링 접점 (Würth WE-SECF 계열 등)</t>
         </is>
       </c>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>공통모드 초크 2×1 mH, ≥0.3 A</t>
+          <t>PCB 가장자리 → 하우징 내면 샤시 접촉 (구 M12 쉘 핀 대체)</t>
         </is>
       </c>
       <c r="J27" s="19" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="L27" s="20">
         <f>D27*J27</f>
@@ -2793,9 +2793,9 @@
         <f>D27*K27</f>
         <v/>
       </c>
-      <c r="N27" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N27" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -2805,12 +2805,12 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
@@ -2818,34 +2818,34 @@
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>22uH</t>
+          <t>CMC 2x1mH 0.3A</t>
         </is>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
-          <t>L_4x4mm</t>
+          <t>CMC_WE-SL</t>
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>Coilcraft</t>
+          <t>Würth</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>XGL4030-223ME (확인)</t>
+          <t>WE-SL2 계열 (품번 확인)</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
         <is>
-          <t>파워 인덕터 22 uH, 4×4 mm, Isat ≥ 0.8 A</t>
+          <t>공통모드 초크 2×1 mH, ≥0.3 A</t>
         </is>
       </c>
       <c r="J28" s="19" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="K28" s="19" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="L28" s="20">
         <f>D28*J28</f>
@@ -2867,12 +2867,12 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="D29" s="18" t="n">
@@ -2880,34 +2880,34 @@
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>4.7R 1W pulse</t>
+          <t>22uH</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>R_MELF_MMB-0207</t>
+          <t>L_4x4mm</t>
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Coilcraft</t>
         </is>
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>MMB 0207 4.7 Ω (품번 확인)</t>
+          <t>XGL4030-223ME (확인)</t>
         </is>
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>MELF 펄스 저항 4.7 Ω 1 W (입력 직렬)</t>
+          <t>파워 인덕터 22 uH, 4×4 mm, Isat ≥ 0.8 A</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="L29" s="20">
         <f>D29*J29</f>
@@ -2929,12 +2929,12 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
@@ -2942,34 +2942,34 @@
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>4.7R 1W pulse</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_MELF_MMB-0207</t>
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>MMB 0207 4.7 Ω (품번 확인)</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>저항 1 MΩ 1% 0603</t>
+          <t>MELF 펄스 저항 4.7 Ω 1 W (입력 직렬)</t>
         </is>
       </c>
       <c r="J30" s="19" t="n">
-        <v>0.002</v>
+        <v>0.1</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.005</v>
+        <v>0.3</v>
       </c>
       <c r="L30" s="20">
         <f>D30*J30</f>
@@ -2979,9 +2979,9 @@
         <f>D30*K30</f>
         <v/>
       </c>
-      <c r="N30" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N30" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -2991,12 +2991,12 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="D31" s="18" t="n">
@@ -3004,7 +3004,7 @@
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>866k 1%</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
@@ -3019,12 +3019,12 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07866KL</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>저항 866 kΩ 1% 0603 (UVLO)</t>
+          <t>저항 1 MΩ 1% 0603</t>
         </is>
       </c>
       <c r="J31" s="19" t="n">
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="D32" s="18" t="n">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>97.6k 1%</t>
+          <t>866k 1%</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
@@ -3081,12 +3081,12 @@
       </c>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0797K6L</t>
+          <t>RC0603FR-07866KL</t>
         </is>
       </c>
       <c r="I32" s="17" t="inlineStr">
         <is>
-          <t>저항 97.6 kΩ 1% 0603 (UVLO/OVP)</t>
+          <t>저항 866 kΩ 1% 0603 (UVLO)</t>
         </is>
       </c>
       <c r="J32" s="19" t="n">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="D33" s="18" t="n">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>36.5k 1%</t>
+          <t>97.6k 1%</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
@@ -3143,12 +3143,12 @@
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0736K5L</t>
+          <t>RC0603FR-0797K6L</t>
         </is>
       </c>
       <c r="I33" s="17" t="inlineStr">
         <is>
-          <t>저항 36.5 kΩ 1% 0603 (OVP)</t>
+          <t>저항 97.6 kΩ 1% 0603 (UVLO/OVP)</t>
         </is>
       </c>
       <c r="J33" s="19" t="n">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>R_ILIM *</t>
+          <t>36.5k 1%</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
@@ -3205,12 +3205,12 @@
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07 (값 TBD)</t>
+          <t>RC0603FR-0736K5L</t>
         </is>
       </c>
       <c r="I34" s="17" t="inlineStr">
         <is>
-          <t>저항 1% 0603 — TPS2660 전류제한 150 mA 값 계산 필요</t>
+          <t>저항 36.5 kΩ 1% 0603 (OVP)</t>
         </is>
       </c>
       <c r="J34" s="19" t="n">
@@ -3227,9 +3227,9 @@
         <f>D34*K34</f>
         <v/>
       </c>
-      <c r="N34" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N34" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3239,20 +3239,20 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>R7 R11 R12 R13 R14 R15 R31 R41</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="D35" s="18" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>R_ILIM *</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
@@ -3267,12 +3267,12 @@
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-07 (값 TBD)</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>저항 10 kΩ 1% 0603</t>
+          <t>저항 1% 0603 — TPS2660 전류제한 150 mA 값 계산 필요</t>
         </is>
       </c>
       <c r="J35" s="19" t="n">
@@ -3289,9 +3289,9 @@
         <f>D35*K35</f>
         <v/>
       </c>
-      <c r="N35" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N35" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -3301,20 +3301,20 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R7 R11 R12 R13 R14 R15 R31 R41</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="I36" s="17" t="inlineStr">
         <is>
-          <t>저항 100 kΩ 1% 0603 (벅 FB)</t>
+          <t>저항 10 kΩ 1% 0603</t>
         </is>
       </c>
       <c r="J36" s="19" t="n">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="D37" s="18" t="n">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>24.9k 1%</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
@@ -3391,12 +3391,12 @@
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0724K9L</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>저항 24.9 kΩ 1% 0603 (벅 FB)</t>
+          <t>저항 100 kΩ 1% 0603 (벅 FB)</t>
         </is>
       </c>
       <c r="J37" s="19" t="n">
@@ -3425,20 +3425,20 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>R16 R17 R18 R20</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>24.9k 1%</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
@@ -3453,12 +3453,12 @@
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-071KL</t>
+          <t>RC0603FR-0724K9L</t>
         </is>
       </c>
       <c r="I38" s="17" t="inlineStr">
         <is>
-          <t>저항 1 kΩ 1% 0603</t>
+          <t>저항 24.9 kΩ 1% 0603 (벅 FB)</t>
         </is>
       </c>
       <c r="J38" s="19" t="n">
@@ -3487,20 +3487,20 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R16 R17 R18 R20</t>
         </is>
       </c>
       <c r="D39" s="18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>4.02k 0.01% 5ppm</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
@@ -3510,24 +3510,24 @@
       </c>
       <c r="G39" s="16" t="inlineStr">
         <is>
-          <t>Vishay / Susumu</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>0.01% 5 ppm 박막 (품번 확인)</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="I39" s="17" t="inlineStr">
         <is>
-          <t>Pt1000 기준저항 4.02 kΩ 0.01% 5 ppm/K 0603</t>
+          <t>저항 1 kΩ 1% 0603</t>
         </is>
       </c>
       <c r="J39" s="19" t="n">
-        <v>1</v>
+        <v>0.002</v>
       </c>
       <c r="K39" s="19" t="n">
-        <v>4</v>
+        <v>0.005</v>
       </c>
       <c r="L39" s="20">
         <f>D39*J39</f>
@@ -3537,9 +3537,9 @@
         <f>D39*K39</f>
         <v/>
       </c>
-      <c r="N39" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N39" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3549,12 +3549,12 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
@@ -3562,7 +3562,7 @@
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>0R RTN link*</t>
+          <t>4.02k 0.01% 5ppm</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
@@ -3572,24 +3572,24 @@
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Vishay / Susumu</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>RC0603JR-070RL</t>
+          <t>0.01% 5 ppm 박막 (품번 확인)</t>
         </is>
       </c>
       <c r="I40" s="17" t="inlineStr">
         <is>
-          <t>0 Ω 링크 — TPS2660 RTN 연결 확인 후 실장 여부 결정</t>
+          <t>Pt1000 기준저항 4.02 kΩ 0.01% 5 ppm/K 0603</t>
         </is>
       </c>
       <c r="J40" s="19" t="n">
-        <v>0.002</v>
+        <v>1</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>0.005</v>
+        <v>4</v>
       </c>
       <c r="L40" s="20">
         <f>D40*J40</f>
@@ -3611,47 +3611,47 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>R30 R40</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="D41" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>10R pulse</t>
+          <t>0R RTN link*</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>CRCW251210R0FKEGHP (확인)</t>
+          <t>RC0603JR-070RL</t>
         </is>
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>펄스 내성 저항 10 Ω 2512 (출력 직렬)</t>
+          <t>0 Ω 링크 — TPS2660 RTN 연결 확인 후 실장 여부 결정</t>
         </is>
       </c>
       <c r="J41" s="19" t="n">
-        <v>0.05</v>
+        <v>0.002</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>0.15</v>
+        <v>0.005</v>
       </c>
       <c r="L41" s="20">
         <f>D41*J41</f>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>R60 R61</t>
+          <t>R30 R40</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
@@ -3686,34 +3686,34 @@
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>2.2R (or 0R)</t>
+          <t>10R pulse</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="H42" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-072R2L</t>
+          <t>CRCW251210R0FKEGHP (확인)</t>
         </is>
       </c>
       <c r="I42" s="17" t="inlineStr">
         <is>
-          <t>저항 2.2 Ω 1% 0603 (RS-485 직렬)</t>
+          <t>펄스 내성 저항 10 Ω 2512 (출력 직렬)</t>
         </is>
       </c>
       <c r="J42" s="19" t="n">
-        <v>0.002</v>
+        <v>0.05</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>0.005</v>
+        <v>0.15</v>
       </c>
       <c r="L42" s="20">
         <f>D42*J42</f>
@@ -3723,9 +3723,9 @@
         <f>D42*K42</f>
         <v/>
       </c>
-      <c r="N42" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N42" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -3735,47 +3735,47 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R60 R61</t>
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>2.2R (or 0R)</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>RC0603FR-072R2L</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
+          <t>저항 2.2 Ω 1% 0603 (RS-485 직렬)</t>
         </is>
       </c>
       <c r="J43" s="19" t="n">
-        <v>1.5</v>
+        <v>0.002</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>3</v>
+        <v>0.005</v>
       </c>
       <c r="L43" s="20">
         <f>D43*J43</f>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="N43" s="16" t="inlineStr">
         <is>
-          <t>확정</t>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
@@ -3810,12 +3810,12 @@
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>LMR36006</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>VQFN-HR-12_LMR36006</t>
+          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
         </is>
       </c>
       <c r="G44" s="16" t="inlineStr">
@@ -3825,19 +3825,19 @@
       </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>LMR36006 (가변판 주문코드 확인)</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="I44" s="17" t="inlineStr">
         <is>
-          <t>벅 60 V 0.6 A → 5 V</t>
+          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
         </is>
       </c>
       <c r="J44" s="19" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="L44" s="20">
         <f>D44*J44</f>
@@ -3847,9 +3847,9 @@
         <f>D44*K44</f>
         <v/>
       </c>
-      <c r="N44" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N44" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="D45" s="18" t="n">
@@ -3872,12 +3872,12 @@
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>LMR36006</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>VQFN-HR-12_LMR36006</t>
         </is>
       </c>
       <c r="G45" s="16" t="inlineStr">
@@ -3887,19 +3887,19 @@
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>LMR36006 (가변판 주문코드 확인)</t>
         </is>
       </c>
       <c r="I45" s="17" t="inlineStr">
         <is>
-          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
+          <t>벅 60 V 0.6 A → 5 V</t>
         </is>
       </c>
       <c r="J45" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>1</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
       <c r="L45" s="20">
         <f>D45*J45</f>
@@ -3909,9 +3909,9 @@
         <f>D45*K45</f>
         <v/>
       </c>
-      <c r="N45" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N45" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3921,12 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
@@ -3934,34 +3934,34 @@
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>LQFP-48_7x7mm_P0.5mm</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="G46" s="16" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="I46" s="17" t="inlineStr">
         <is>
-          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
+          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
         </is>
       </c>
       <c r="J46" s="19" t="n">
-        <v>1.5</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
       <c r="L46" s="20">
         <f>D46*J46</f>
@@ -3983,12 +3983,12 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="D47" s="18" t="n">
@@ -3996,34 +3996,34 @@
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>QFN-24_PCAP04</t>
+          <t>LQFP-48_7x7mm_P0.5mm</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>ScioSense</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>정전용량-디지털 변환기 QFN24</t>
+          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
         </is>
       </c>
       <c r="J47" s="19" t="n">
-        <v>6.5</v>
+        <v>1.5</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>7.1</v>
+        <v>2.5</v>
       </c>
       <c r="L47" s="20">
         <f>D47*J47</f>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
@@ -4058,34 +4058,34 @@
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
+          <t>QFN-24_PCAP04</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>ScioSense</t>
         </is>
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="I48" s="17" t="inlineStr">
         <is>
-          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
+          <t>정전용량-디지털 변환기 QFN24</t>
         </is>
       </c>
       <c r="J48" s="19" t="n">
-        <v>1.9</v>
+        <v>6.5</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>3.5</v>
+        <v>7.1</v>
       </c>
       <c r="L48" s="20">
         <f>D48*J48</f>
@@ -4107,25 +4107,25 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>U7 U8</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="D49" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>DAC8760IPWP</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>HTSSOP-24_DAC8760</t>
+          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
@@ -4135,19 +4135,19 @@
       </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>DAC8760IPWPR</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="I49" s="17" t="inlineStr">
         <is>
-          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
+          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
         </is>
       </c>
       <c r="J49" s="19" t="n">
-        <v>7.8</v>
+        <v>1.9</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>12.4</v>
+        <v>3.5</v>
       </c>
       <c r="L49" s="20">
         <f>D49*J49</f>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>U9 U10</t>
+          <t>U7 U8</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
@@ -4182,12 +4182,12 @@
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>DAC8760IPWP</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>HTSSOP-24_DAC8760</t>
         </is>
       </c>
       <c r="G50" s="16" t="inlineStr">
@@ -4197,19 +4197,19 @@
       </c>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>TPS26611 (패키지·주문코드 확인)</t>
+          <t>DAC8760IPWPR</t>
         </is>
       </c>
       <c r="I50" s="17" t="inlineStr">
         <is>
-          <t>4–20 mA 출력 오결선 보호</t>
+          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
         </is>
       </c>
       <c r="J50" s="19" t="n">
-        <v>1.2</v>
+        <v>7.8</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>2.5</v>
+        <v>12.4</v>
       </c>
       <c r="L50" s="20">
         <f>D50*J50</f>
@@ -4219,9 +4219,9 @@
         <f>D50*K50</f>
         <v/>
       </c>
-      <c r="N50" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N50" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -4231,25 +4231,25 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>통신</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U9 U10</t>
         </is>
       </c>
       <c r="D51" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
@@ -4259,19 +4259,19 @@
       </c>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>TPS26611 (패키지·주문코드 확인)</t>
         </is>
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
+          <t>4–20 mA 출력 오결선 보호</t>
         </is>
       </c>
       <c r="J51" s="19" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L51" s="20">
         <f>D51*J51</f>
@@ -4281,9 +4281,9 @@
         <f>D51*K51</f>
         <v/>
       </c>
-      <c r="N51" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N51" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4293,12 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>기판</t>
+          <t>통신</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
@@ -4306,34 +4306,34 @@
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>HMT500-E-301</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="I52" s="17" t="inlineStr">
         <is>
-          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
+          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
         </is>
       </c>
       <c r="J52" s="19" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L52" s="20">
         <f>D52*J52</f>
@@ -4343,9 +4343,9 @@
         <f>D52*K52</f>
         <v/>
       </c>
-      <c r="N52" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N52" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -4355,12 +4355,12 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>기판</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>센서 헤드</t>
+          <t>PCB</t>
         </is>
       </c>
       <c r="D53" s="18" t="n">
@@ -4378,24 +4378,24 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>IST</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>MK33-W mini (150138)</t>
+          <t>HMT500-E-301</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
         <is>
-          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
+          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
         </is>
       </c>
       <c r="J53" s="19" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="K53" s="19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L53" s="20">
         <f>D53*J53</f>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="N53" s="21" t="inlineStr">
         <is>
-          <t>사내 단가</t>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4445,19 +4445,19 @@
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>MiniSens Pt1000 F0.1</t>
+          <t>MK33-W mini (150138)</t>
         </is>
       </c>
       <c r="I54" s="17" t="inlineStr">
         <is>
-          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
+          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J54" s="19" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L54" s="20">
         <f>D54*J54</f>
@@ -4469,7 +4469,7 @@
       </c>
       <c r="N54" s="21" t="inlineStr">
         <is>
-          <t>추정</t>
+          <t>사내 단가</t>
         </is>
       </c>
     </row>
@@ -4479,12 +4479,12 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>센서 헤드</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
@@ -4502,24 +4502,24 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>SHR-04V-S</t>
+          <t>MiniSens Pt1000 F0.1</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
         <is>
-          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
+          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J55" s="19" t="n">
-        <v>0.04</v>
+        <v>0.5</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>0.1</v>
+        <v>3</v>
       </c>
       <c r="L55" s="20">
         <f>D55*J55</f>
@@ -4529,9 +4529,9 @@
         <f>D55*K55</f>
         <v/>
       </c>
-      <c r="N55" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N55" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4541,16 +4541,16 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>P-204</t>
         </is>
       </c>
       <c r="D56" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
@@ -4564,24 +4564,24 @@
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>M Connect</t>
         </is>
       </c>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>TBD (두텍 사용품)</t>
         </is>
       </c>
       <c r="I56" s="17" t="inlineStr">
         <is>
-          <t>SH 크림프 단자 AWG 32–28</t>
+          <t>M12 8핀 수컷 전면 장착형 M16×1.5, 리드선형 (W-2 납땜)</t>
         </is>
       </c>
       <c r="J56" s="19" t="n">
-        <v>0.03</v>
+        <v>2</v>
       </c>
       <c r="K56" s="19" t="n">
-        <v>0.06</v>
+        <v>10</v>
       </c>
       <c r="L56" s="20">
         <f>D56*J56</f>
@@ -4591,9 +4591,9 @@
         <f>D56*K56</f>
         <v/>
       </c>
-      <c r="N56" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N56" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D57" s="18" t="n">
@@ -4626,24 +4626,24 @@
       </c>
       <c r="G57" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>PTFE AWG30 전선</t>
+          <t>GHR-08V-S</t>
         </is>
       </c>
       <c r="I57" s="17" t="inlineStr">
         <is>
-          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
+          <t>GH 1.25 mm 8핀 소켓 하우징 (M12 하네스 W-2)</t>
         </is>
       </c>
       <c r="J57" s="19" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="K57" s="19" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="L57" s="20">
         <f>D57*J57</f>
@@ -4653,9 +4653,9 @@
         <f>D57*K57</f>
         <v/>
       </c>
-      <c r="N57" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N57" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -4665,47 +4665,47 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>조립</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
+          <t>W-2</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="E58" s="16" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D58" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="16" t="inlineStr">
+      <c r="F58" s="16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F58" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G58" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>SMT 양면 실장</t>
+          <t>SSHL-002T-P0.2</t>
         </is>
       </c>
       <c r="I58" s="17" t="inlineStr">
         <is>
-          <t>1k 기준 조립비</t>
+          <t>GH 크림프 단자 AWG 30–26</t>
         </is>
       </c>
       <c r="J58" s="19" t="n">
-        <v>2</v>
+        <v>0.03</v>
       </c>
       <c r="K58" s="19" t="n">
-        <v>4</v>
+        <v>0.06</v>
       </c>
       <c r="L58" s="20">
         <f>D58*J58</f>
@@ -4715,24 +4715,334 @@
         <f>D58*K58</f>
         <v/>
       </c>
-      <c r="N58" s="21" t="inlineStr">
+      <c r="N58" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>W-2</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G59" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" s="17" t="inlineStr">
+        <is>
+          <t>PTFE AWG28 전선</t>
+        </is>
+      </c>
+      <c r="I59" s="17" t="inlineStr">
+        <is>
+          <t>UL1213 계열 200 °C, 8심 × 60 mm + 수축튜브 (M12 핀 납땜)</t>
+        </is>
+      </c>
+      <c r="J59" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K59" s="19" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L59" s="20">
+        <f>D59*J59</f>
+        <v/>
+      </c>
+      <c r="M59" s="20">
+        <f>D59*K59</f>
+        <v/>
+      </c>
+      <c r="N59" s="21" t="inlineStr">
         <is>
           <t>추정</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="I59" s="3" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="16" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G60" s="16" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="H60" s="17" t="inlineStr">
+        <is>
+          <t>SHR-04V-S</t>
+        </is>
+      </c>
+      <c r="I60" s="17" t="inlineStr">
+        <is>
+          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
+        </is>
+      </c>
+      <c r="J60" s="19" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K60" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L60" s="20">
+        <f>D60*J60</f>
+        <v/>
+      </c>
+      <c r="M60" s="20">
+        <f>D60*K60</f>
+        <v/>
+      </c>
+      <c r="N60" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G61" s="16" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="H61" s="17" t="inlineStr">
+        <is>
+          <t>SSH-003T-P0.2-H</t>
+        </is>
+      </c>
+      <c r="I61" s="17" t="inlineStr">
+        <is>
+          <t>SH 크림프 단자 AWG 32–28</t>
+        </is>
+      </c>
+      <c r="J61" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K61" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L61" s="20">
+        <f>D61*J61</f>
+        <v/>
+      </c>
+      <c r="M61" s="20">
+        <f>D61*K61</f>
+        <v/>
+      </c>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" s="17" t="inlineStr">
+        <is>
+          <t>PTFE AWG30 전선</t>
+        </is>
+      </c>
+      <c r="I62" s="17" t="inlineStr">
+        <is>
+          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
+        </is>
+      </c>
+      <c r="J62" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K62" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L62" s="20">
+        <f>D62*J62</f>
+        <v/>
+      </c>
+      <c r="M62" s="20">
+        <f>D62*K62</f>
+        <v/>
+      </c>
+      <c r="N62" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>조립</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H63" s="17" t="inlineStr">
+        <is>
+          <t>SMT 양면 실장</t>
+        </is>
+      </c>
+      <c r="I63" s="17" t="inlineStr">
+        <is>
+          <t>1k 기준 조립비</t>
+        </is>
+      </c>
+      <c r="J63" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L63" s="20">
+        <f>D63*J63</f>
+        <v/>
+      </c>
+      <c r="M63" s="20">
+        <f>D63*K63</f>
+        <v/>
+      </c>
+      <c r="N63" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="I64" s="3" t="inlineStr">
         <is>
           <t>합계 (1대분)</t>
         </is>
       </c>
-      <c r="L59" s="23">
-        <f>SUM(L2:L58)</f>
-        <v/>
-      </c>
-      <c r="M59" s="23">
-        <f>SUM(M2:M58)</f>
+      <c r="L64" s="23">
+        <f>SUM(L2:L63)</f>
+        <v/>
+      </c>
+      <c r="M64" s="23">
+        <f>SUM(M2:M63)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
J3 sensor header to right-angle JST SH SM04B-SRSS-TB
- Side entry facing the sensor (-x) at PCB x 22.5-26.5, height 2.95; W-1 plugs
  in straight from the holder hole with no bend
- PCAP04 / ADS1220 / Cref moved behind J3
- Schematic footprint, parts list, board zone label, CAD, drawings, renders,
  docs, decision log #19 and tests updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA2o8uJsqp9Vzsg4b665ev
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500/HMT500_parts_list.xlsx
+++ b/hardware/kicad/HMT500/HMT500_parts_list.xlsx
@@ -2694,12 +2694,12 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>BM04B-SRSS-TB</t>
+          <t>SM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
-          <t>JST_SH_BM04B-SRSS-TB_1x04-1MP_P1.00mm_Vertical</t>
+          <t>JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
@@ -2709,12 +2709,12 @@
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>BM04B-SRSS-TB</t>
+          <t>SM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>SH 1.0 mm 4핀 헤더, 윗면 삽입 SMD (센서 하네스 W-1, 정격 −25~+85 °C)</t>
+          <t>SH 1.0 mm 4핀 헤더, 옆 삽입(직각) SMD (센서 하네스 W-1, 정격 −25~+85 °C)</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">

</xml_diff>

<commit_message>
Schematic v0.6: parts cleanup (91 -> 75) and PCB temperature sensing
- Removed: fault pull-ups R11-R15 (MCU internal pull-ups), status LED D3/R16
  (not visible after potting), RS-485 R60/R61/D60/D61 (THVD2450 built-in
  protection), VREF+ filter FB2/C19 (MCU ADC only for diagnostics), C11/C2/C6
  (duplicated by adjacent capacitors); VREF+ tied to +3V3 with C20
- PCB temperature with no added parts: ADS1220 internal sensor at the measurement
  front, STM32G0 internal sensor mid-board; compensation plan in circuit-design 5B
- 63 nets, netlist check 0 errors; parts list regenerated; decision log #22/#23

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA2o8uJsqp9Vzsg4b665ev
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500/HMT500_parts_list.xlsx
+++ b/hardware/kicad/HMT500/HMT500_parts_list.xlsx
@@ -262,8 +262,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N63" headerRowCount="1">
-  <autoFilter ref="A1:N63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N60" headerRowCount="1">
+  <autoFilter ref="A1:N60"/>
   <tableColumns count="14">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="분류"/>
@@ -573,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -652,15 +652,15 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A7)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A7)</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A7)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A7)</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A7)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A7)</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -679,15 +679,15 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A8)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A8)</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A8)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A8)</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A8)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A8)</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -706,15 +706,15 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A9)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A9)</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A9)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A9)</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A9)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A9)</f>
         <v/>
       </c>
       <c r="E9" s="10">
@@ -729,19 +729,19 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>표시</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="B10" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A10)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A10)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A10)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A10)</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A10)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A10)</f>
         <v/>
       </c>
       <c r="E10" s="10">
@@ -756,19 +756,19 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>커넥터</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A11)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A11)</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A11)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A11)</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A11)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A11)</f>
         <v/>
       </c>
       <c r="E11" s="10">
@@ -783,19 +783,19 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>생산</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A12)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A12)</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A12)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A12)</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A12)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A12)</f>
         <v/>
       </c>
       <c r="E12" s="10">
@@ -810,19 +810,19 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A13)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A13)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A13)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A13)</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A13)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A13)</f>
         <v/>
       </c>
       <c r="E13" s="10">
@@ -837,19 +837,19 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="B14" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A14)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A14)</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A14)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A14)</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A14)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A14)</f>
         <v/>
       </c>
       <c r="E14" s="10">
@@ -864,19 +864,19 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>통신</t>
         </is>
       </c>
       <c r="B15" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A15)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A15)</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A15)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A15)</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A15)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A15)</f>
         <v/>
       </c>
       <c r="E15" s="10">
@@ -891,19 +891,19 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>통신</t>
+          <t>기판</t>
         </is>
       </c>
       <c r="B16" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A16)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A16)</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A16)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A16)</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A16)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A16)</f>
         <v/>
       </c>
       <c r="E16" s="10">
@@ -918,19 +918,19 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>기판</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="B17" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A17)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A17)</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A17)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A17)</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A17)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A17)</f>
         <v/>
       </c>
       <c r="E17" s="10">
@@ -945,19 +945,19 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A18)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A18)</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A18)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A18)</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A18)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A18)</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -972,19 +972,19 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>조립</t>
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A19)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$60,A19)</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A19)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A19)</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A19)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A19)</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -997,89 +997,62 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>조립</t>
-        </is>
-      </c>
-      <c r="B20" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$63,A20)</f>
-        <v/>
-      </c>
-      <c r="C20" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A20)</f>
-        <v/>
-      </c>
-      <c r="D20" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A20)</f>
-        <v/>
-      </c>
-      <c r="E20" s="10">
-        <f>C20*$B$4</f>
-        <v/>
-      </c>
-      <c r="F20" s="10">
-        <f>D20*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="B21" s="11">
-        <f>SUM(B7:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="12">
-        <f>SUM(C7:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="12">
-        <f>SUM(D7:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="13">
-        <f>SUM(E7:E20)</f>
-        <v/>
-      </c>
-      <c r="F21" s="13">
-        <f>SUM(F7:F20)</f>
-        <v/>
+      <c r="B20" s="11">
+        <f>SUM(B7:B19)</f>
+        <v/>
+      </c>
+      <c r="C20" s="12">
+        <f>SUM(C7:C19)</f>
+        <v/>
+      </c>
+      <c r="D20" s="12">
+        <f>SUM(D7:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="13">
+        <f>SUM(E7:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="13">
+        <f>SUM(F7:F19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>읽는 법</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>읽는 법</t>
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>· 부품리스트 시트의 참조번호·수량·값·풋프린트는 KiCad 회로도에서 자동 생성 (make_parts_list.py).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>· 부품리스트 시트의 참조번호·수량·값·풋프린트는 KiCad 회로도에서 자동 생성 (make_parts_list.py).</t>
+          <t>· 상태: 확정 = 회로도·품번 확정 / 제안 = 동등품 대체 가능 / 확인 필요 = 데이터시트·견적 확인 후 확정 / TBD = 미정.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>· 상태: 확정 = 회로도·품번 확정 / 제안 = 동등품 대체 가능 / 확인 필요 = 데이터시트·견적 확인 후 확정 / TBD = 미정.</t>
+          <t>· 제외: 기구 부품(바디·하우징·캡·엔드캡·홀더·O링·나사), 피드스루(HMT500-P-201)는 기구 부품표에 있음.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>· 제외: 기구 부품(바디·하우징·캡·엔드캡·홀더·O링·나사), 피드스루(HMT500-P-201)는 기구 부품표에 있음.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>· 핀 번호 확인 대상 IC: LMR36006, PCAP04, DAC8760, TPS26611 (회로도 VERIFY 표시). TPS2660은 R22 RTN 연결 확인.</t>
         </is>
@@ -1096,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N64"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1198,11 +1171,11 @@
       </c>
       <c r="C2" s="17" t="inlineStr">
         <is>
-          <t>C1 C6</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="D2" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
@@ -1255,25 +1228,25 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>C2 C5</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="D3" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>10u 50V</t>
+          <t>4.7n 2kV Y2</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>C_1210_3225Metric</t>
+          <t>C_1812_4532Metric</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
@@ -1283,19 +1256,19 @@
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>GRM32ER71H106KA12L</t>
+          <t>GA343QR7GF472KW01L</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
         <is>
-          <t>MLCC 10 uF 50 V X7R 1210</t>
+          <t>Safety cap 4.7 nF Y2 (250 VAC) 1812</t>
         </is>
       </c>
       <c r="J3" s="19" t="n">
         <v>0.15</v>
       </c>
       <c r="K3" s="19" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="L3" s="20">
         <f>D3*J3</f>
@@ -1317,12 +1290,12 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C4" s="17" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="D4" s="18" t="n">
@@ -1330,12 +1303,12 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>4.7n 2kV Y2</t>
+          <t>22n</t>
         </is>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>C_1812_4532Metric</t>
+          <t>C_0603_1608Metric</t>
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr">
@@ -1345,19 +1318,19 @@
       </c>
       <c r="H4" s="17" t="inlineStr">
         <is>
-          <t>GA343QR7GF472KW01L</t>
+          <t>GRM188R71H223KA01D</t>
         </is>
       </c>
       <c r="I4" s="17" t="inlineStr">
         <is>
-          <t>Safety cap 4.7 nF Y2 (250 VAC) 1812</t>
+          <t>MLCC 22 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="J4" s="19" t="n">
-        <v>0.15</v>
+        <v>0.004</v>
       </c>
       <c r="K4" s="19" t="n">
-        <v>0.4</v>
+        <v>0.01</v>
       </c>
       <c r="L4" s="20">
         <f>D4*J4</f>
@@ -1384,7 +1357,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="D5" s="18" t="n">
@@ -1392,12 +1365,12 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>22n</t>
+          <t>10u 50V</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>C_0603_1608Metric</t>
+          <t>C_1210_3225Metric</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
@@ -1407,19 +1380,19 @@
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>GRM188R71H223KA01D</t>
+          <t>GRM32ER71H106KA12L</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>MLCC 22 nF 50 V X7R 0603</t>
+          <t>MLCC 10 uF 50 V X7R 1210</t>
         </is>
       </c>
       <c r="J5" s="19" t="n">
-        <v>0.004</v>
+        <v>0.15</v>
       </c>
       <c r="K5" s="19" t="n">
-        <v>0.01</v>
+        <v>0.35</v>
       </c>
       <c r="L5" s="20">
         <f>D5*J5</f>
@@ -1570,11 +1543,11 @@
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>C9 C11 C12 C19 C24 C25 C26</t>
+          <t>C9 C12 C24 C25 C26</t>
         </is>
       </c>
       <c r="D8" s="18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
@@ -2247,47 +2220,47 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>표시</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D30 D40</t>
         </is>
       </c>
       <c r="D19" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="16" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>SMAJ33CA</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>LED_0603_1608Metric</t>
+          <t>D_SMA</t>
         </is>
       </c>
       <c r="G19" s="16" t="inlineStr">
         <is>
-          <t>Würth</t>
+          <t>Littelfuse</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>150060GS75000</t>
+          <t>SMAJ33CA</t>
         </is>
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>LED 녹색 0603</t>
+          <t>TVS 400 W 33 V 양방향 SMA (아날로그 출력)</t>
         </is>
       </c>
       <c r="J19" s="19" t="n">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
       <c r="K19" s="19" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="L19" s="20">
         <f>D19*J19</f>
@@ -2309,47 +2282,47 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>D30 D40</t>
+          <t>FB1</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E20" s="16" t="inlineStr">
         <is>
-          <t>SMAJ33CA</t>
+          <t>600R@100MHz</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>L_0603_1608Metric</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>SMAJ33CA</t>
+          <t>BLM18KG601SN1D</t>
         </is>
       </c>
       <c r="I20" s="17" t="inlineStr">
         <is>
-          <t>TVS 400 W 33 V 양방향 SMA (아날로그 출력)</t>
+          <t>페라이트 비드 600 Ω@100 MHz 0603</t>
         </is>
       </c>
       <c r="J20" s="19" t="n">
-        <v>0.06</v>
+        <v>0.01</v>
       </c>
       <c r="K20" s="19" t="n">
-        <v>0.15</v>
+        <v>0.03</v>
       </c>
       <c r="L20" s="20">
         <f>D20*J20</f>
@@ -2376,42 +2349,42 @@
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>D60 D61</t>
+          <t>GDT1</t>
         </is>
       </c>
       <c r="D21" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="16" t="inlineStr">
         <is>
-          <t>SMAJ40CA (opt.)</t>
+          <t>GDT 230V</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
-          <t>D_SMA</t>
+          <t>GDT_Bourns_2038</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
-          <t>Littelfuse</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>SMAJ40CA</t>
+          <t>2038-23-SM-RPLF</t>
         </is>
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>TVS 400 W 40 V 양방향 SMA (RS-485, 옵션)</t>
+          <t>GDT 230 V SMD (회로 GND–외함)</t>
         </is>
       </c>
       <c r="J21" s="19" t="n">
-        <v>0.06</v>
+        <v>0.4</v>
       </c>
       <c r="K21" s="19" t="n">
-        <v>0.15</v>
+        <v>1</v>
       </c>
       <c r="L21" s="20">
         <f>D21*J21</f>
@@ -2421,9 +2394,9 @@
         <f>D21*K21</f>
         <v/>
       </c>
-      <c r="N21" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N21" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -2433,47 +2406,47 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>FB1 FB2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="D22" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" s="16" t="inlineStr">
         <is>
-          <t>600R@100MHz</t>
+          <t>SM08B-GHS-TB</t>
         </is>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
-          <t>L_0603_1608Metric</t>
+          <t>JST_GH_SM08B-GHS-TB_1x08-1MP_P1.25mm_Horizontal</t>
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H22" s="17" t="inlineStr">
         <is>
-          <t>BLM18KG601SN1D</t>
+          <t>SM08B-GHS-TB</t>
         </is>
       </c>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>페라이트 비드 600 Ω@100 MHz 0603</t>
+          <t>GH 1.25 mm 8핀 헤더, 옆 삽입(직각) SMD (M12 하네스 W-2, 정격 −25~+85 °C)</t>
         </is>
       </c>
       <c r="J22" s="19" t="n">
-        <v>0.01</v>
+        <v>0.35</v>
       </c>
       <c r="K22" s="19" t="n">
-        <v>0.03</v>
+        <v>0.8</v>
       </c>
       <c r="L22" s="20">
         <f>D22*J22</f>
@@ -2495,12 +2468,12 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>생산</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>GDT1</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="D23" s="18" t="n">
@@ -2508,34 +2481,34 @@
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>GDT 230V</t>
+          <t>TC2030-IDC-NL</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
-          <t>GDT_Bourns_2038</t>
+          <t>Tag-Connect_TC2030-IDC-NL_2x03_P1.27mm_Vertical</t>
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Tag-Connect</t>
         </is>
       </c>
       <c r="H23" s="17" t="inlineStr">
         <is>
-          <t>2038-23-SM-RPLF</t>
+          <t>(PCB 패드만)</t>
         </is>
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>GDT 230 V SMD (회로 GND–외함)</t>
+          <t>SWD 기록용 패드 — 부품 실장 없음</t>
         </is>
       </c>
       <c r="J23" s="19" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="K23" s="19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" s="20">
         <f>D23*J23</f>
@@ -2545,9 +2518,9 @@
         <f>D23*K23</f>
         <v/>
       </c>
-      <c r="N23" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2535,7 @@
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="D24" s="18" t="n">
@@ -2570,12 +2543,12 @@
       </c>
       <c r="E24" s="16" t="inlineStr">
         <is>
-          <t>SM08B-GHS-TB</t>
+          <t>SM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
-          <t>JST_GH_SM08B-GHS-TB_1x08-1MP_P1.25mm_Horizontal</t>
+          <t>JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</t>
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr">
@@ -2585,19 +2558,19 @@
       </c>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>SM08B-GHS-TB</t>
+          <t>SM04B-SRSS-TB</t>
         </is>
       </c>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>GH 1.25 mm 8핀 헤더, 옆 삽입(직각) SMD (M12 하네스 W-2, 정격 −25~+85 °C)</t>
+          <t>SH 1.0 mm 4핀 헤더, 옆 삽입(직각) SMD (센서 하네스 W-1, 정격 −25~+85 °C)</t>
         </is>
       </c>
       <c r="J24" s="19" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="K24" s="19" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L24" s="20">
         <f>D24*J24</f>
@@ -2619,12 +2592,12 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>생산</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J5</t>
         </is>
       </c>
       <c r="D25" s="18" t="n">
@@ -2632,34 +2605,34 @@
       </c>
       <c r="E25" s="16" t="inlineStr">
         <is>
-          <t>TC2030-IDC-NL</t>
+          <t>Chassis contact</t>
         </is>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
-          <t>Tag-Connect_TC2030-IDC-NL_2x03_P1.27mm_Vertical</t>
+          <t>Chassis_Spring_Contact</t>
         </is>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
-          <t>Tag-Connect</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>(PCB 패드만)</t>
+          <t>SMD 스프링 접점 (Würth WE-SECF 계열 등)</t>
         </is>
       </c>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>SWD 기록용 패드 — 부품 실장 없음</t>
+          <t>PCB 가장자리 → 하우징 내면 샤시 접촉 (구 M12 쉘 핀 대체)</t>
         </is>
       </c>
       <c r="J25" s="19" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="K25" s="19" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="L25" s="20">
         <f>D25*J25</f>
@@ -2669,9 +2642,9 @@
         <f>D25*K25</f>
         <v/>
       </c>
-      <c r="N25" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N25" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -2681,12 +2654,12 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>커넥터</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="D26" s="18" t="n">
@@ -2694,34 +2667,34 @@
       </c>
       <c r="E26" s="16" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB</t>
+          <t>CMC 2x1mH 0.3A</t>
         </is>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
-          <t>JST_SH_SM04B-SRSS-TB_1x04-1MP_P1.00mm_Horizontal</t>
+          <t>CMC_WE-SL</t>
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Würth</t>
         </is>
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB</t>
+          <t>WE-SL2 계열 (품번 확인)</t>
         </is>
       </c>
       <c r="I26" s="17" t="inlineStr">
         <is>
-          <t>SH 1.0 mm 4핀 헤더, 옆 삽입(직각) SMD (센서 하네스 W-1, 정격 −25~+85 °C)</t>
+          <t>공통모드 초크 2×1 mH, ≥0.3 A</t>
         </is>
       </c>
       <c r="J26" s="19" t="n">
         <v>0.3</v>
       </c>
       <c r="K26" s="19" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="L26" s="20">
         <f>D26*J26</f>
@@ -2731,9 +2704,9 @@
         <f>D26*K26</f>
         <v/>
       </c>
-      <c r="N26" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N26" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -2743,12 +2716,12 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>커넥터</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="D27" s="18" t="n">
@@ -2756,34 +2729,34 @@
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>Chassis contact</t>
+          <t>22uH</t>
         </is>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
-          <t>Chassis_Spring_Contact</t>
+          <t>L_4x4mm</t>
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Coilcraft</t>
         </is>
       </c>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>SMD 스프링 접점 (Würth WE-SECF 계열 등)</t>
+          <t>XGL4030-223ME (확인)</t>
         </is>
       </c>
       <c r="I27" s="17" t="inlineStr">
         <is>
-          <t>PCB 가장자리 → 하우징 내면 샤시 접촉 (구 M12 쉘 핀 대체)</t>
+          <t>파워 인덕터 22 uH, 4×4 mm, Isat ≥ 0.8 A</t>
         </is>
       </c>
       <c r="J27" s="19" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="K27" s="19" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="L27" s="20">
         <f>D27*J27</f>
@@ -2793,9 +2766,9 @@
         <f>D27*K27</f>
         <v/>
       </c>
-      <c r="N27" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N27" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2783,7 @@
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
@@ -2818,34 +2791,34 @@
       </c>
       <c r="E28" s="16" t="inlineStr">
         <is>
-          <t>CMC 2x1mH 0.3A</t>
+          <t>4.7R 1W pulse</t>
         </is>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
-          <t>CMC_WE-SL</t>
+          <t>R_MELF_MMB-0207</t>
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
         <is>
-          <t>Würth</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>WE-SL2 계열 (품번 확인)</t>
+          <t>MMB 0207 4.7 Ω (품번 확인)</t>
         </is>
       </c>
       <c r="I28" s="17" t="inlineStr">
         <is>
-          <t>공통모드 초크 2×1 mH, ≥0.3 A</t>
+          <t>MELF 펄스 저항 4.7 Ω 1 W (입력 직렬)</t>
         </is>
       </c>
       <c r="J28" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K28" s="19" t="n">
         <v>0.3</v>
-      </c>
-      <c r="K28" s="19" t="n">
-        <v>0.8</v>
       </c>
       <c r="L28" s="20">
         <f>D28*J28</f>
@@ -2867,12 +2840,12 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="D29" s="18" t="n">
@@ -2880,34 +2853,34 @@
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>22uH</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>L_4x4mm</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
-          <t>Coilcraft</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>XGL4030-223ME (확인)</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="I29" s="17" t="inlineStr">
         <is>
-          <t>파워 인덕터 22 uH, 4×4 mm, Isat ≥ 0.8 A</t>
+          <t>저항 1 MΩ 1% 0603</t>
         </is>
       </c>
       <c r="J29" s="19" t="n">
-        <v>0.25</v>
+        <v>0.002</v>
       </c>
       <c r="K29" s="19" t="n">
-        <v>0.6</v>
+        <v>0.005</v>
       </c>
       <c r="L29" s="20">
         <f>D29*J29</f>
@@ -2917,9 +2890,9 @@
         <f>D29*K29</f>
         <v/>
       </c>
-      <c r="N29" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N29" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -2929,12 +2902,12 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="D30" s="18" t="n">
@@ -2942,34 +2915,34 @@
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>4.7R 1W pulse</t>
+          <t>866k 1%</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>R_MELF_MMB-0207</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>MMB 0207 4.7 Ω (품번 확인)</t>
+          <t>RC0603FR-07866KL</t>
         </is>
       </c>
       <c r="I30" s="17" t="inlineStr">
         <is>
-          <t>MELF 펄스 저항 4.7 Ω 1 W (입력 직렬)</t>
+          <t>저항 866 kΩ 1% 0603 (UVLO)</t>
         </is>
       </c>
       <c r="J30" s="19" t="n">
-        <v>0.1</v>
+        <v>0.002</v>
       </c>
       <c r="K30" s="19" t="n">
-        <v>0.3</v>
+        <v>0.005</v>
       </c>
       <c r="L30" s="20">
         <f>D30*J30</f>
@@ -2979,9 +2952,9 @@
         <f>D30*K30</f>
         <v/>
       </c>
-      <c r="N30" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N30" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -2991,12 +2964,12 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="D31" s="18" t="n">
@@ -3004,7 +2977,7 @@
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>97.6k 1%</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
@@ -3019,12 +2992,12 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>RC0603FR-0797K6L</t>
         </is>
       </c>
       <c r="I31" s="17" t="inlineStr">
         <is>
-          <t>저항 1 MΩ 1% 0603</t>
+          <t>저항 97.6 kΩ 1% 0603 (UVLO/OVP)</t>
         </is>
       </c>
       <c r="J31" s="19" t="n">
@@ -3058,7 +3031,7 @@
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="D32" s="18" t="n">
@@ -3066,7 +3039,7 @@
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>866k 1%</t>
+          <t>36.5k 1%</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
@@ -3081,12 +3054,12 @@
       </c>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07866KL</t>
+          <t>RC0603FR-0736K5L</t>
         </is>
       </c>
       <c r="I32" s="17" t="inlineStr">
         <is>
-          <t>저항 866 kΩ 1% 0603 (UVLO)</t>
+          <t>저항 36.5 kΩ 1% 0603 (OVP)</t>
         </is>
       </c>
       <c r="J32" s="19" t="n">
@@ -3120,7 +3093,7 @@
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R6</t>
         </is>
       </c>
       <c r="D33" s="18" t="n">
@@ -3128,7 +3101,7 @@
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>97.6k 1%</t>
+          <t>R_ILIM *</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
@@ -3143,12 +3116,12 @@
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0797K6L</t>
+          <t>RC0603FR-07 (값 TBD)</t>
         </is>
       </c>
       <c r="I33" s="17" t="inlineStr">
         <is>
-          <t>저항 97.6 kΩ 1% 0603 (UVLO/OVP)</t>
+          <t>저항 1% 0603 — TPS2660 전류제한 150 mA 값 계산 필요</t>
         </is>
       </c>
       <c r="J33" s="19" t="n">
@@ -3165,9 +3138,9 @@
         <f>D33*K33</f>
         <v/>
       </c>
-      <c r="N33" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N33" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -3177,20 +3150,20 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R7 R31 R41</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>36.5k 1%</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
@@ -3205,12 +3178,12 @@
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0736K5L</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="I34" s="17" t="inlineStr">
         <is>
-          <t>저항 36.5 kΩ 1% 0603 (OVP)</t>
+          <t>저항 10 kΩ 1% 0603</t>
         </is>
       </c>
       <c r="J34" s="19" t="n">
@@ -3244,7 +3217,7 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="D35" s="18" t="n">
@@ -3252,7 +3225,7 @@
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>R_ILIM *</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
@@ -3267,12 +3240,12 @@
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07 (값 TBD)</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>저항 1% 0603 — TPS2660 전류제한 150 mA 값 계산 필요</t>
+          <t>저항 100 kΩ 1% 0603 (벅 FB)</t>
         </is>
       </c>
       <c r="J35" s="19" t="n">
@@ -3289,9 +3262,9 @@
         <f>D35*K35</f>
         <v/>
       </c>
-      <c r="N35" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N35" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3301,20 +3274,20 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>R7 R11 R12 R13 R14 R15 R31 R41</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>24.9k 1%</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
@@ -3329,12 +3302,12 @@
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-0724K9L</t>
         </is>
       </c>
       <c r="I36" s="17" t="inlineStr">
         <is>
-          <t>저항 10 kΩ 1% 0603</t>
+          <t>저항 24.9 kΩ 1% 0603 (벅 FB)</t>
         </is>
       </c>
       <c r="J36" s="19" t="n">
@@ -3363,20 +3336,20 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R17 R18 R20</t>
         </is>
       </c>
       <c r="D37" s="18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
@@ -3391,12 +3364,12 @@
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>저항 100 kΩ 1% 0603 (벅 FB)</t>
+          <t>저항 1 kΩ 1% 0603</t>
         </is>
       </c>
       <c r="J37" s="19" t="n">
@@ -3425,12 +3398,12 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="D38" s="18" t="n">
@@ -3438,7 +3411,7 @@
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>24.9k 1%</t>
+          <t>4.02k 0.01% 5ppm</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
@@ -3448,24 +3421,24 @@
       </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Vishay / Susumu</t>
         </is>
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-0724K9L</t>
+          <t>0.01% 5 ppm 박막 (품번 확인)</t>
         </is>
       </c>
       <c r="I38" s="17" t="inlineStr">
         <is>
-          <t>저항 24.9 kΩ 1% 0603 (벅 FB)</t>
+          <t>Pt1000 기준저항 4.02 kΩ 0.01% 5 ppm/K 0603</t>
         </is>
       </c>
       <c r="J38" s="19" t="n">
-        <v>0.002</v>
+        <v>1</v>
       </c>
       <c r="K38" s="19" t="n">
-        <v>0.005</v>
+        <v>4</v>
       </c>
       <c r="L38" s="20">
         <f>D38*J38</f>
@@ -3475,9 +3448,9 @@
         <f>D38*K38</f>
         <v/>
       </c>
-      <c r="N38" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N38" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -3487,20 +3460,20 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>수동</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>R16 R17 R18 R20</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="D39" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>0R RTN link*</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
@@ -3515,12 +3488,12 @@
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-071KL</t>
+          <t>RC0603JR-070RL</t>
         </is>
       </c>
       <c r="I39" s="17" t="inlineStr">
         <is>
-          <t>저항 1 kΩ 1% 0603</t>
+          <t>0 Ω 링크 — TPS2660 RTN 연결 확인 후 실장 여부 결정</t>
         </is>
       </c>
       <c r="J39" s="19" t="n">
@@ -3537,9 +3510,9 @@
         <f>D39*K39</f>
         <v/>
       </c>
-      <c r="N39" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N39" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -3549,47 +3522,47 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>보호</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R30 R40</t>
         </is>
       </c>
       <c r="D40" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>4.02k 0.01% 5ppm</t>
+          <t>10R pulse</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>R_2512_6332Metric</t>
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr">
         <is>
-          <t>Vishay / Susumu</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>0.01% 5 ppm 박막 (품번 확인)</t>
+          <t>CRCW251210R0FKEGHP (확인)</t>
         </is>
       </c>
       <c r="I40" s="17" t="inlineStr">
         <is>
-          <t>Pt1000 기준저항 4.02 kΩ 0.01% 5 ppm/K 0603</t>
+          <t>펄스 내성 저항 10 Ω 2512 (출력 직렬)</t>
         </is>
       </c>
       <c r="J40" s="19" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="K40" s="19" t="n">
-        <v>4</v>
+        <v>0.15</v>
       </c>
       <c r="L40" s="20">
         <f>D40*J40</f>
@@ -3616,7 +3589,7 @@
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="D41" s="18" t="n">
@@ -3624,34 +3597,34 @@
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>0R RTN link*</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>RC0603JR-070RL</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>0 Ω 링크 — TPS2660 RTN 연결 확인 후 실장 여부 결정</t>
+          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
         </is>
       </c>
       <c r="J41" s="19" t="n">
-        <v>0.002</v>
+        <v>1.5</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>0.005</v>
+        <v>3</v>
       </c>
       <c r="L41" s="20">
         <f>D41*J41</f>
@@ -3661,9 +3634,9 @@
         <f>D41*K41</f>
         <v/>
       </c>
-      <c r="N41" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N41" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -3673,47 +3646,47 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>R30 R40</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>10R pulse</t>
+          <t>LMR36006</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>R_2512_6332Metric</t>
+          <t>VQFN-HR-12_LMR36006</t>
         </is>
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H42" s="17" t="inlineStr">
         <is>
-          <t>CRCW251210R0FKEGHP (확인)</t>
+          <t>LMR36006 (가변판 주문코드 확인)</t>
         </is>
       </c>
       <c r="I42" s="17" t="inlineStr">
         <is>
-          <t>펄스 내성 저항 10 Ω 2512 (출력 직렬)</t>
+          <t>벅 60 V 0.6 A → 5 V</t>
         </is>
       </c>
       <c r="J42" s="19" t="n">
-        <v>0.05</v>
+        <v>1</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>0.15</v>
+        <v>1.6</v>
       </c>
       <c r="L42" s="20">
         <f>D42*J42</f>
@@ -3735,47 +3708,47 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>보호</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>R60 R61</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="D43" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>2.2R (or 0R)</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>R_0603_1608Metric</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>RC0603FR-072R2L</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>저항 2.2 Ω 1% 0603 (RS-485 직렬)</t>
+          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
         </is>
       </c>
       <c r="J43" s="19" t="n">
-        <v>0.002</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>0.005</v>
+        <v>0.3</v>
       </c>
       <c r="L43" s="20">
         <f>D43*J43</f>
@@ -3787,7 +3760,7 @@
       </c>
       <c r="N43" s="16" t="inlineStr">
         <is>
-          <t>제안</t>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -3797,12 +3770,12 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
@@ -3810,34 +3783,34 @@
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
+          <t>LQFP-48_7x7mm_P0.5mm</t>
         </is>
       </c>
       <c r="G44" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="I44" s="17" t="inlineStr">
         <is>
-          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
+          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
         </is>
       </c>
       <c r="J44" s="19" t="n">
         <v>1.5</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="L44" s="20">
         <f>D44*J44</f>
@@ -3859,12 +3832,12 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="D45" s="18" t="n">
@@ -3872,34 +3845,34 @@
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>LMR36006</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>VQFN-HR-12_LMR36006</t>
+          <t>QFN-24_PCAP04</t>
         </is>
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>ScioSense</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>LMR36006 (가변판 주문코드 확인)</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="I45" s="17" t="inlineStr">
         <is>
-          <t>벅 60 V 0.6 A → 5 V</t>
+          <t>정전용량-디지털 변환기 QFN24</t>
         </is>
       </c>
       <c r="J45" s="19" t="n">
-        <v>1</v>
+        <v>6.5</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>1.6</v>
+        <v>7.1</v>
       </c>
       <c r="L45" s="20">
         <f>D45*J45</f>
@@ -3909,9 +3882,9 @@
         <f>D45*K45</f>
         <v/>
       </c>
-      <c r="N45" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N45" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3894,12 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
@@ -3934,12 +3907,12 @@
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
         </is>
       </c>
       <c r="G46" s="16" t="inlineStr">
@@ -3949,19 +3922,19 @@
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="I46" s="17" t="inlineStr">
         <is>
-          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
+          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
         </is>
       </c>
       <c r="J46" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.9</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>0.3</v>
+        <v>3.5</v>
       </c>
       <c r="L46" s="20">
         <f>D46*J46</f>
@@ -3983,47 +3956,47 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U7 U8</t>
         </is>
       </c>
       <c r="D47" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>DAC8760IPWP</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>LQFP-48_7x7mm_P0.5mm</t>
+          <t>HTSSOP-24_DAC8760</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>DAC8760IPWPR</t>
         </is>
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
+          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
         </is>
       </c>
       <c r="J47" s="19" t="n">
-        <v>1.5</v>
+        <v>7.8</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>2.5</v>
+        <v>12.4</v>
       </c>
       <c r="L47" s="20">
         <f>D47*J47</f>
@@ -4045,47 +4018,47 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U9 U10</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>QFN-24_PCAP04</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
         <is>
-          <t>ScioSense</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>TPS26611 (패키지·주문코드 확인)</t>
         </is>
       </c>
       <c r="I48" s="17" t="inlineStr">
         <is>
-          <t>정전용량-디지털 변환기 QFN24</t>
+          <t>4–20 mA 출력 오결선 보호</t>
         </is>
       </c>
       <c r="J48" s="19" t="n">
-        <v>6.5</v>
+        <v>1.2</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>7.1</v>
+        <v>2.5</v>
       </c>
       <c r="L48" s="20">
         <f>D48*J48</f>
@@ -4095,9 +4068,9 @@
         <f>D48*K48</f>
         <v/>
       </c>
-      <c r="N48" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N48" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -4107,12 +4080,12 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>통신</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="D49" s="18" t="n">
@@ -4120,12 +4093,12 @@
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
@@ -4135,19 +4108,19 @@
       </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="I49" s="17" t="inlineStr">
         <is>
-          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
+          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
         </is>
       </c>
       <c r="J49" s="19" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="L49" s="20">
         <f>D49*J49</f>
@@ -4169,47 +4142,47 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>기판</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>U7 U8</t>
+          <t>PCB</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H50" s="17" t="inlineStr">
+        <is>
+          <t>HMT500-E-301</t>
+        </is>
+      </c>
+      <c r="I50" s="17" t="inlineStr">
+        <is>
+          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
+        </is>
+      </c>
+      <c r="J50" s="19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K50" s="19" t="n">
         <v>2</v>
-      </c>
-      <c r="E50" s="16" t="inlineStr">
-        <is>
-          <t>DAC8760IPWP</t>
-        </is>
-      </c>
-      <c r="F50" s="16" t="inlineStr">
-        <is>
-          <t>HTSSOP-24_DAC8760</t>
-        </is>
-      </c>
-      <c r="G50" s="16" t="inlineStr">
-        <is>
-          <t>TI</t>
-        </is>
-      </c>
-      <c r="H50" s="17" t="inlineStr">
-        <is>
-          <t>DAC8760IPWPR</t>
-        </is>
-      </c>
-      <c r="I50" s="17" t="inlineStr">
-        <is>
-          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
-        </is>
-      </c>
-      <c r="J50" s="19" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="K50" s="19" t="n">
-        <v>12.4</v>
       </c>
       <c r="L50" s="20">
         <f>D50*J50</f>
@@ -4219,9 +4192,9 @@
         <f>D50*K50</f>
         <v/>
       </c>
-      <c r="N50" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N50" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4231,47 +4204,47 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>U9 U10</t>
+          <t>센서 헤드</t>
         </is>
       </c>
       <c r="D51" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>TPS26611 (패키지·주문코드 확인)</t>
+          <t>MK33-W mini (150138)</t>
         </is>
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>4–20 mA 출력 오결선 보호</t>
+          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J51" s="19" t="n">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="L51" s="20">
         <f>D51*J51</f>
@@ -4283,7 +4256,7 @@
       </c>
       <c r="N51" s="21" t="inlineStr">
         <is>
-          <t>확인 필요</t>
+          <t>사내 단가</t>
         </is>
       </c>
     </row>
@@ -4293,12 +4266,12 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>통신</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>센서 헤드</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
@@ -4306,31 +4279,31 @@
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>MiniSens Pt1000 F0.1</t>
         </is>
       </c>
       <c r="I52" s="17" t="inlineStr">
         <is>
-          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
+          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J52" s="19" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="K52" s="19" t="n">
         <v>3</v>
@@ -4343,9 +4316,9 @@
         <f>D52*K52</f>
         <v/>
       </c>
-      <c r="N52" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N52" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4355,12 +4328,12 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>기판</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>P-204</t>
         </is>
       </c>
       <c r="D53" s="18" t="n">
@@ -4378,24 +4351,24 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>M Connect</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>HMT500-E-301</t>
+          <t>TBD (두텍 사용품)</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
         <is>
-          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
+          <t>M12 8핀 수컷 전면 장착형 M16×1.5, 리드선형 (W-2 납땜)</t>
         </is>
       </c>
       <c r="J53" s="19" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="K53" s="19" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="L53" s="20">
         <f>D53*J53</f>
@@ -4405,9 +4378,9 @@
         <f>D53*K53</f>
         <v/>
       </c>
-      <c r="N53" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N53" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -4417,12 +4390,12 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>센서 헤드</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
@@ -4440,24 +4413,24 @@
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>IST</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>MK33-W mini (150138)</t>
+          <t>GHR-08V-S</t>
         </is>
       </c>
       <c r="I54" s="17" t="inlineStr">
         <is>
-          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
+          <t>GH 1.25 mm 8핀 소켓 하우징 (M12 하네스 W-2)</t>
         </is>
       </c>
       <c r="J54" s="19" t="n">
-        <v>0</v>
+        <v>0.06</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="L54" s="20">
         <f>D54*J54</f>
@@ -4467,9 +4440,9 @@
         <f>D54*K54</f>
         <v/>
       </c>
-      <c r="N54" s="21" t="inlineStr">
-        <is>
-          <t>사내 단가</t>
+      <c r="N54" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -4479,16 +4452,16 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>센서 헤드</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
@@ -4502,24 +4475,24 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>IST</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>MiniSens Pt1000 F0.1</t>
+          <t>SSHL-002T-P0.2</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
         <is>
-          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
+          <t>GH 크림프 단자 AWG 30–26</t>
         </is>
       </c>
       <c r="J55" s="19" t="n">
-        <v>0.5</v>
+        <v>0.03</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>3</v>
+        <v>0.06</v>
       </c>
       <c r="L55" s="20">
         <f>D55*J55</f>
@@ -4529,9 +4502,9 @@
         <f>D55*K55</f>
         <v/>
       </c>
-      <c r="N55" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N55" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -4541,12 +4514,12 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>커넥터</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>P-204</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D56" s="18" t="n">
@@ -4564,24 +4537,24 @@
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>M Connect</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>TBD (두텍 사용품)</t>
+          <t>PTFE AWG28 전선</t>
         </is>
       </c>
       <c r="I56" s="17" t="inlineStr">
         <is>
-          <t>M12 8핀 수컷 전면 장착형 M16×1.5, 리드선형 (W-2 납땜)</t>
+          <t>UL1213 계열 200 °C, 8심 × 60 mm + 수축튜브 (M12 핀 납땜)</t>
         </is>
       </c>
       <c r="J56" s="19" t="n">
-        <v>2</v>
+        <v>0.15</v>
       </c>
       <c r="K56" s="19" t="n">
-        <v>10</v>
+        <v>0.4</v>
       </c>
       <c r="L56" s="20">
         <f>D56*J56</f>
@@ -4591,9 +4564,9 @@
         <f>D56*K56</f>
         <v/>
       </c>
-      <c r="N56" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N56" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4581,7 @@
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>W-1</t>
         </is>
       </c>
       <c r="D57" s="18" t="n">
@@ -4631,19 +4604,19 @@
       </c>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>GHR-08V-S</t>
+          <t>SHR-04V-S</t>
         </is>
       </c>
       <c r="I57" s="17" t="inlineStr">
         <is>
-          <t>GH 1.25 mm 8핀 소켓 하우징 (M12 하네스 W-2)</t>
+          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
         </is>
       </c>
       <c r="J57" s="19" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="K57" s="19" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="L57" s="20">
         <f>D57*J57</f>
@@ -4670,11 +4643,11 @@
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>W-1</t>
         </is>
       </c>
       <c r="D58" s="18" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
@@ -4693,12 +4666,12 @@
       </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>SSHL-002T-P0.2</t>
+          <t>SSH-003T-P0.2-H</t>
         </is>
       </c>
       <c r="I58" s="17" t="inlineStr">
         <is>
-          <t>GH 크림프 단자 AWG 30–26</t>
+          <t>SH 크림프 단자 AWG 32–28</t>
         </is>
       </c>
       <c r="J58" s="19" t="n">
@@ -4732,7 +4705,7 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>W-1</t>
         </is>
       </c>
       <c r="D59" s="18" t="n">
@@ -4755,19 +4728,19 @@
       </c>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>PTFE AWG28 전선</t>
+          <t>PTFE AWG30 전선</t>
         </is>
       </c>
       <c r="I59" s="17" t="inlineStr">
         <is>
-          <t>UL1213 계열 200 °C, 8심 × 60 mm + 수축튜브 (M12 핀 납땜)</t>
+          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
         </is>
       </c>
       <c r="J59" s="19" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="K59" s="19" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L59" s="20">
         <f>D59*J59</f>
@@ -4789,12 +4762,12 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>조립</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D60" s="18" t="n">
@@ -4812,24 +4785,24 @@
       </c>
       <c r="G60" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>SHR-04V-S</t>
+          <t>SMT 양면 실장</t>
         </is>
       </c>
       <c r="I60" s="17" t="inlineStr">
         <is>
-          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
+          <t>1k 기준 조립비</t>
         </is>
       </c>
       <c r="J60" s="19" t="n">
-        <v>0.04</v>
+        <v>2</v>
       </c>
       <c r="K60" s="19" t="n">
-        <v>0.1</v>
+        <v>4</v>
       </c>
       <c r="L60" s="20">
         <f>D60*J60</f>
@@ -4839,210 +4812,24 @@
         <f>D60*K60</f>
         <v/>
       </c>
-      <c r="N60" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N60" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="16" t="inlineStr">
-        <is>
-          <t>하네스</t>
-        </is>
-      </c>
-      <c r="C61" s="17" t="inlineStr">
-        <is>
-          <t>W-1</t>
-        </is>
-      </c>
-      <c r="D61" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E61" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="16" t="inlineStr">
-        <is>
-          <t>JST</t>
-        </is>
-      </c>
-      <c r="H61" s="17" t="inlineStr">
-        <is>
-          <t>SSH-003T-P0.2-H</t>
-        </is>
-      </c>
-      <c r="I61" s="17" t="inlineStr">
-        <is>
-          <t>SH 크림프 단자 AWG 32–28</t>
-        </is>
-      </c>
-      <c r="J61" s="19" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="K61" s="19" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="L61" s="20">
-        <f>D61*J61</f>
-        <v/>
-      </c>
-      <c r="M61" s="20">
-        <f>D61*K61</f>
-        <v/>
-      </c>
-      <c r="N61" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="16" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="16" t="inlineStr">
-        <is>
-          <t>하네스</t>
-        </is>
-      </c>
-      <c r="C62" s="17" t="inlineStr">
-        <is>
-          <t>W-1</t>
-        </is>
-      </c>
-      <c r="D62" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F62" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G62" s="16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H62" s="17" t="inlineStr">
-        <is>
-          <t>PTFE AWG30 전선</t>
-        </is>
-      </c>
-      <c r="I62" s="17" t="inlineStr">
-        <is>
-          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
-        </is>
-      </c>
-      <c r="J62" s="19" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K62" s="19" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="L62" s="20">
-        <f>D62*J62</f>
-        <v/>
-      </c>
-      <c r="M62" s="20">
-        <f>D62*K62</f>
-        <v/>
-      </c>
-      <c r="N62" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
-        <is>
-          <t>조립</t>
-        </is>
-      </c>
-      <c r="C63" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D63" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G63" s="16" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H63" s="17" t="inlineStr">
-        <is>
-          <t>SMT 양면 실장</t>
-        </is>
-      </c>
-      <c r="I63" s="17" t="inlineStr">
-        <is>
-          <t>1k 기준 조립비</t>
-        </is>
-      </c>
-      <c r="J63" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="K63" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="L63" s="20">
-        <f>D63*J63</f>
-        <v/>
-      </c>
-      <c r="M63" s="20">
-        <f>D63*K63</f>
-        <v/>
-      </c>
-      <c r="N63" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="I64" s="3" t="inlineStr">
+      <c r="I61" s="3" t="inlineStr">
         <is>
           <t>합계 (1대분)</t>
         </is>
       </c>
-      <c r="L64" s="23">
-        <f>SUM(L2:L63)</f>
-        <v/>
-      </c>
-      <c r="M64" s="23">
-        <f>SUM(M2:M63)</f>
+      <c r="L61" s="23">
+        <f>SUM(L2:L60)</f>
+        <v/>
+      </c>
+      <c r="M61" s="23">
+        <f>SUM(M2:M60)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Schematic v0.7: DAC8760 real pinout, OPA197 +VSENSE buffer, ISET-R, SPI2 daisy chain
- DAC8760 symbol from datasheet SBAS528D (HTSSOP-24 PWP + EP), same as
  VibrationSensor IVS320; placeholder pins removed, VERIFY flag dropped
- +VSENSE via OPA197 unity-gain follower (U12/U13) of the terminal voltage;
  R31/R41 10k kept as buffer input protection; C45/C55 V+ bypass
- External ISET-R 15k 0.1% 25 ppm (R32/R42)
- DACs on dedicated SPI2 (PB13/14/15) daisy chain with common DAC_LATCH
  (PB10); R33 100k pull-down on DAC_DAISY; ALARM -> PB11/PB3, PWR_FLT -> PB4
- Output protection unification (TPS26611 vs passive) left on hold
- Parts list, circuit-design doc, decision log #24 updated; netlist 70/70, 0 errors

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JA2o8uJsqp9Vzsg4b665ev
</commit_message>
<xml_diff>
--- a/hardware/kicad/HMT500/HMT500_parts_list.xlsx
+++ b/hardware/kicad/HMT500/HMT500_parts_list.xlsx
@@ -262,8 +262,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N60" headerRowCount="1">
-  <autoFilter ref="A1:N60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PartsList" displayName="PartsList" ref="A1:N63" headerRowCount="1">
+  <autoFilter ref="A1:N63"/>
   <tableColumns count="14">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="분류"/>
@@ -652,15 +652,15 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A7)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="C7" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A7)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="D7" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A7)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A7)</f>
         <v/>
       </c>
       <c r="E7" s="10">
@@ -679,15 +679,15 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A8)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A8)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A8)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A8)</f>
         <v/>
       </c>
       <c r="E8" s="10">
@@ -706,15 +706,15 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A9)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A9)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A9)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A9)</f>
         <v/>
       </c>
       <c r="E9" s="10">
@@ -733,15 +733,15 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A10)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="C10" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A10)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="D10" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A10)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A10)</f>
         <v/>
       </c>
       <c r="E10" s="10">
@@ -760,15 +760,15 @@
         </is>
       </c>
       <c r="B11" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A11)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="C11" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A11)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A11)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A11)</f>
         <v/>
       </c>
       <c r="E11" s="10">
@@ -787,15 +787,15 @@
         </is>
       </c>
       <c r="B12" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A12)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="C12" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A12)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="D12" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A12)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A12)</f>
         <v/>
       </c>
       <c r="E12" s="10">
@@ -810,19 +810,19 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="B13" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A13)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="C13" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A13)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="D13" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A13)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A13)</f>
         <v/>
       </c>
       <c r="E13" s="10">
@@ -837,19 +837,19 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="B14" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A14)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A14)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A14)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A14)</f>
         <v/>
       </c>
       <c r="E14" s="10">
@@ -868,15 +868,15 @@
         </is>
       </c>
       <c r="B15" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A15)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A15)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A15)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A15)</f>
         <v/>
       </c>
       <c r="E15" s="10">
@@ -895,15 +895,15 @@
         </is>
       </c>
       <c r="B16" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A16)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="C16" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A16)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="D16" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A16)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A16)</f>
         <v/>
       </c>
       <c r="E16" s="10">
@@ -922,15 +922,15 @@
         </is>
       </c>
       <c r="B17" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A17)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="C17" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A17)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="D17" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A17)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A17)</f>
         <v/>
       </c>
       <c r="E17" s="10">
@@ -949,15 +949,15 @@
         </is>
       </c>
       <c r="B18" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A18)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A18)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A18)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A18)</f>
         <v/>
       </c>
       <c r="E18" s="10">
@@ -976,15 +976,15 @@
         </is>
       </c>
       <c r="B19" s="8">
-        <f>COUNTIF('부품리스트'!$B$2:$B$60,A19)</f>
+        <f>COUNTIF('부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS('부품리스트'!$L$2:$L$60,'부품리스트'!$B$2:$B$60,A19)</f>
+        <f>SUMIFS('부품리스트'!$L$2:$L$63,'부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>SUMIFS('부품리스트'!$M$2:$M$60,'부품리스트'!$B$2:$B$60,A19)</f>
+        <f>SUMIFS('부품리스트'!$M$2:$M$63,'부품리스트'!$B$2:$B$63,A19)</f>
         <v/>
       </c>
       <c r="E19" s="10">
@@ -1054,7 +1054,7 @@
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>· 핀 번호 확인 대상 IC: LMR36006, PCAP04, DAC8760, TPS26611 (회로도 VERIFY 표시). TPS2660은 R22 RTN 연결 확인.</t>
+          <t>· 핀 번호 확인 대상 IC: LMR36006, PCAP04, TPS26611 (회로도 VERIFY 표시; DAC8760은 v0.7에서 데이터시트 핀 확정). TPS2660은 R22 RTN 연결 확인.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N61"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1977,11 +1977,11 @@
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>C42 C52</t>
+          <t>C42 C45 C52 C55</t>
         </is>
       </c>
       <c r="D15" s="18" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
@@ -3584,47 +3584,47 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R32 R42</t>
         </is>
       </c>
       <c r="D41" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>15k 0.1% 25ppm</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G41" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>TPS26600PWPR</t>
+          <t>RT0603BRD0715KL</t>
         </is>
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
+          <t>저항 15 kΩ 0.1% 25 ppm/K 0603 (DAC8760 외부 ISET-R)</t>
         </is>
       </c>
       <c r="J41" s="19" t="n">
-        <v>1.5</v>
+        <v>0.02</v>
       </c>
       <c r="K41" s="19" t="n">
-        <v>3</v>
+        <v>0.06</v>
       </c>
       <c r="L41" s="20">
         <f>D41*J41</f>
@@ -3636,7 +3636,7 @@
       </c>
       <c r="N41" s="16" t="inlineStr">
         <is>
-          <t>확정</t>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3646,12 +3646,12 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>전원</t>
+          <t>수동</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
@@ -3659,34 +3659,34 @@
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>LMR36006</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>VQFN-HR-12_LMR36006</t>
+          <t>R_0603_1608Metric</t>
         </is>
       </c>
       <c r="G42" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="H42" s="17" t="inlineStr">
         <is>
-          <t>LMR36006 (가변판 주문코드 확인)</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="I42" s="17" t="inlineStr">
         <is>
-          <t>벅 60 V 0.6 A → 5 V</t>
+          <t>저항 100 kΩ 1% 0603 (DAC 데이지 체인 풀다운)</t>
         </is>
       </c>
       <c r="J42" s="19" t="n">
-        <v>1</v>
+        <v>0.002</v>
       </c>
       <c r="K42" s="19" t="n">
-        <v>1.6</v>
+        <v>0.005</v>
       </c>
       <c r="L42" s="20">
         <f>D42*J42</f>
@@ -3696,9 +3696,9 @@
         <f>D42*K42</f>
         <v/>
       </c>
-      <c r="N42" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N42" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="D43" s="18" t="n">
@@ -3721,12 +3721,12 @@
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>HTSSOP-16-1EP_4.4x5mm_P0.65mm_EP3.4x5mm_Mask2.66x2.46mm_ThermalVias</t>
         </is>
       </c>
       <c r="G43" s="16" t="inlineStr">
@@ -3736,19 +3736,19 @@
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>TPS7A2033PDBVR</t>
+          <t>TPS26600PWPR</t>
         </is>
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
+          <t>eFuse 60 V 2 A, 역극성·OVP·UVLO, HTSSOP-16</t>
         </is>
       </c>
       <c r="J43" s="19" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="K43" s="19" t="n">
-        <v>0.3</v>
+        <v>3</v>
       </c>
       <c r="L43" s="20">
         <f>D43*J43</f>
@@ -3770,12 +3770,12 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>MCU</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
@@ -3783,34 +3783,34 @@
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>LMR36006</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>LQFP-48_7x7mm_P0.5mm</t>
+          <t>VQFN-HR-12_LMR36006</t>
         </is>
       </c>
       <c r="G44" s="16" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>STM32G0B1CCT3</t>
+          <t>LMR36006 (가변판 주문코드 확인)</t>
         </is>
       </c>
       <c r="I44" s="17" t="inlineStr">
         <is>
-          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
+          <t>벅 60 V 0.6 A → 5 V</t>
         </is>
       </c>
       <c r="J44" s="19" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="K44" s="19" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="L44" s="20">
         <f>D44*J44</f>
@@ -3820,9 +3820,9 @@
         <f>D44*K44</f>
         <v/>
       </c>
-      <c r="N44" s="16" t="inlineStr">
-        <is>
-          <t>확정</t>
+      <c r="N44" s="21" t="inlineStr">
+        <is>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -3832,12 +3832,12 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>전원</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="D45" s="18" t="n">
@@ -3845,34 +3845,34 @@
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>QFN-24_PCAP04</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="G45" s="16" t="inlineStr">
         <is>
-          <t>ScioSense</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>PCAP04-AQFM-24</t>
+          <t>TPS7A2033PDBVR</t>
         </is>
       </c>
       <c r="I45" s="17" t="inlineStr">
         <is>
-          <t>정전용량-디지털 변환기 QFN24</t>
+          <t>LDO 3.3 V 300 mA 저잡음 SOT-23-5</t>
         </is>
       </c>
       <c r="J45" s="19" t="n">
-        <v>6.5</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="K45" s="19" t="n">
-        <v>7.1</v>
+        <v>0.3</v>
       </c>
       <c r="L45" s="20">
         <f>D45*J45</f>
@@ -3894,12 +3894,12 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>측정</t>
+          <t>MCU</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="D46" s="18" t="n">
@@ -3907,34 +3907,34 @@
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
+          <t>LQFP-48_7x7mm_P0.5mm</t>
         </is>
       </c>
       <c r="G46" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>ADS1220IPWR</t>
+          <t>STM32G0B1CCT3</t>
         </is>
       </c>
       <c r="I46" s="17" t="inlineStr">
         <is>
-          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
+          <t>MCU Cortex-M0+ 64 MHz 256 KB, LQFP48, −40~125 °C (사내 DP2000 G0B1CCT6 동일 다이)</t>
         </is>
       </c>
       <c r="J46" s="19" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="K46" s="19" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="L46" s="20">
         <f>D46*J46</f>
@@ -3956,47 +3956,47 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>U7 U8</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="D47" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>DAC8760IPWP</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>HTSSOP-24_DAC8760</t>
+          <t>QFN-24_PCAP04</t>
         </is>
       </c>
       <c r="G47" s="16" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>ScioSense</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>DAC8760IPWPR</t>
+          <t>PCAP04-AQFM-24</t>
         </is>
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
+          <t>정전용량-디지털 변환기 QFN24</t>
         </is>
       </c>
       <c r="J47" s="19" t="n">
-        <v>7.8</v>
+        <v>6.5</v>
       </c>
       <c r="K47" s="19" t="n">
-        <v>12.4</v>
+        <v>7.1</v>
       </c>
       <c r="L47" s="20">
         <f>D47*J47</f>
@@ -4018,25 +4018,25 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>출력</t>
+          <t>측정</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>U9 U10</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="D48" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>TPS26611</t>
+          <t>TSSOP-16_4.4x5mm_P0.65mm</t>
         </is>
       </c>
       <c r="G48" s="16" t="inlineStr">
@@ -4046,19 +4046,19 @@
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>TPS26611 (패키지·주문코드 확인)</t>
+          <t>ADS1220IPWR</t>
         </is>
       </c>
       <c r="I48" s="17" t="inlineStr">
         <is>
-          <t>4–20 mA 출력 오결선 보호</t>
+          <t>24-bit ADC, Pt1000 2선 (J3 패드에서 켈빈 분기), TSSOP-16</t>
         </is>
       </c>
       <c r="J48" s="19" t="n">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="K48" s="19" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="L48" s="20">
         <f>D48*J48</f>
@@ -4068,9 +4068,9 @@
         <f>D48*K48</f>
         <v/>
       </c>
-      <c r="N48" s="21" t="inlineStr">
-        <is>
-          <t>확인 필요</t>
+      <c r="N48" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -4080,25 +4080,25 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>통신</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>U7 U8</t>
         </is>
       </c>
       <c r="D49" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>DAC8760IPWP</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
+          <t>HTSSOP-24-1EP_4.4x7.8mm_P0.65mm_EP3.2x5mm</t>
         </is>
       </c>
       <c r="G49" s="16" t="inlineStr">
@@ -4108,19 +4108,19 @@
       </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>THVD2450DR</t>
+          <t>DAC8760IPWPR</t>
         </is>
       </c>
       <c r="I49" s="17" t="inlineStr">
         <is>
-          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
+          <t>16-bit 전압/전류 출력 DAC, HTSSOP-24. 사양 확정 후 같은 핀 대체: DAC7760(12-bit V/I), DAC8750(16-bit 전류), DAC7750(12-bit 전류)</t>
         </is>
       </c>
       <c r="J49" s="19" t="n">
-        <v>1.5</v>
+        <v>7.8</v>
       </c>
       <c r="K49" s="19" t="n">
-        <v>3</v>
+        <v>12.4</v>
       </c>
       <c r="L49" s="20">
         <f>D49*J49</f>
@@ -4142,47 +4142,47 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>기판</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>U9 U10</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TPS26611</t>
         </is>
       </c>
       <c r="G50" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>HMT500-E-301</t>
+          <t>TPS26611 (패키지·주문코드 확인)</t>
         </is>
       </c>
       <c r="I50" s="17" t="inlineStr">
         <is>
-          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
+          <t>4–20 mA 출력 오결선 보호</t>
         </is>
       </c>
       <c r="J50" s="19" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="K50" s="19" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="L50" s="20">
         <f>D50*J50</f>
@@ -4194,7 +4194,7 @@
       </c>
       <c r="N50" s="21" t="inlineStr">
         <is>
-          <t>추정</t>
+          <t>확인 필요</t>
         </is>
       </c>
     </row>
@@ -4204,12 +4204,12 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>통신</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>센서 헤드</t>
+          <t>U11</t>
         </is>
       </c>
       <c r="D51" s="18" t="n">
@@ -4217,34 +4217,34 @@
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SOIC-8_3.9x4.9mm_P1.27mm</t>
         </is>
       </c>
       <c r="G51" s="16" t="inlineStr">
         <is>
-          <t>IST</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>MK33-W mini (150138)</t>
+          <t>THVD2450DR</t>
         </is>
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
+          <t>RS-485 트랜시버, 버스 ±70 V 내성, SOIC-8</t>
         </is>
       </c>
       <c r="J51" s="19" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="K51" s="19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L51" s="20">
         <f>D51*J51</f>
@@ -4254,9 +4254,9 @@
         <f>D51*K51</f>
         <v/>
       </c>
-      <c r="N51" s="21" t="inlineStr">
-        <is>
-          <t>사내 단가</t>
+      <c r="N51" s="16" t="inlineStr">
+        <is>
+          <t>확정</t>
         </is>
       </c>
     </row>
@@ -4266,47 +4266,47 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>센서</t>
+          <t>출력</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>센서 헤드</t>
+          <t>U12 U13</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>OPA197IDBVR</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="G52" s="16" t="inlineStr">
         <is>
-          <t>IST</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>MiniSens Pt1000 F0.1</t>
+          <t>OPA197IDBVR</t>
         </is>
       </c>
       <c r="I52" s="17" t="inlineStr">
         <is>
-          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
+          <t>36 V 레일투레일 연산증폭기 SOT-23-5 — DAC8760 +VSENSE 버퍼 (이득 1)</t>
         </is>
       </c>
       <c r="J52" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="K52" s="19" t="n">
-        <v>3</v>
+        <v>1.1</v>
       </c>
       <c r="L52" s="20">
         <f>D52*J52</f>
@@ -4316,9 +4316,9 @@
         <f>D52*K52</f>
         <v/>
       </c>
-      <c r="N52" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N52" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
         </is>
       </c>
     </row>
@@ -4328,12 +4328,12 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>커넥터</t>
+          <t>기판</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>P-204</t>
+          <t>PCB</t>
         </is>
       </c>
       <c r="D53" s="18" t="n">
@@ -4351,24 +4351,24 @@
       </c>
       <c r="G53" s="16" t="inlineStr">
         <is>
-          <t>M Connect</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>TBD (두텍 사용품)</t>
+          <t>HMT500-E-301</t>
         </is>
       </c>
       <c r="I53" s="17" t="inlineStr">
         <is>
-          <t>M12 8핀 수컷 전면 장착형 M16×1.5, 리드선형 (W-2 납땜)</t>
+          <t>PCB 4층 57×23 mm, FR-4 1.6 t, ENIG (기구 Rev C 외곽)</t>
         </is>
       </c>
       <c r="J53" s="19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K53" s="19" t="n">
         <v>2</v>
-      </c>
-      <c r="K53" s="19" t="n">
-        <v>10</v>
       </c>
       <c r="L53" s="20">
         <f>D53*J53</f>
@@ -4378,9 +4378,9 @@
         <f>D53*K53</f>
         <v/>
       </c>
-      <c r="N53" s="22" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="N53" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4390,12 +4390,12 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>센서 헤드</t>
         </is>
       </c>
       <c r="D54" s="18" t="n">
@@ -4413,24 +4413,24 @@
       </c>
       <c r="G54" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>GHR-08V-S</t>
+          <t>MK33-W mini (150138)</t>
         </is>
       </c>
       <c r="I54" s="17" t="inlineStr">
         <is>
-          <t>GH 1.25 mm 8핀 소켓 하우징 (M12 하네스 W-2)</t>
+          <t>정전용량 습도 소자 200 pF (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J54" s="19" t="n">
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="K54" s="19" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="L54" s="20">
         <f>D54*J54</f>
@@ -4440,9 +4440,9 @@
         <f>D54*K54</f>
         <v/>
       </c>
-      <c r="N54" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N54" s="21" t="inlineStr">
+        <is>
+          <t>사내 단가</t>
         </is>
       </c>
     </row>
@@ -4452,16 +4452,16 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>센서</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>센서 헤드</t>
         </is>
       </c>
       <c r="D55" s="18" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
@@ -4475,24 +4475,24 @@
       </c>
       <c r="G55" s="16" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>IST</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>SSHL-002T-P0.2</t>
+          <t>MiniSens Pt1000 F0.1</t>
         </is>
       </c>
       <c r="I55" s="17" t="inlineStr">
         <is>
-          <t>GH 크림프 단자 AWG 30–26</t>
+          <t>온도 소자 1.6×1.2 mm (센서 프로브 P-202에 실장)</t>
         </is>
       </c>
       <c r="J55" s="19" t="n">
-        <v>0.03</v>
+        <v>0.5</v>
       </c>
       <c r="K55" s="19" t="n">
-        <v>0.06</v>
+        <v>3</v>
       </c>
       <c r="L55" s="20">
         <f>D55*J55</f>
@@ -4502,9 +4502,9 @@
         <f>D55*K55</f>
         <v/>
       </c>
-      <c r="N55" s="16" t="inlineStr">
-        <is>
-          <t>제안</t>
+      <c r="N55" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
         </is>
       </c>
     </row>
@@ -4514,12 +4514,12 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>하네스</t>
+          <t>커넥터</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>P-204</t>
         </is>
       </c>
       <c r="D56" s="18" t="n">
@@ -4537,24 +4537,24 @@
       </c>
       <c r="G56" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>M Connect</t>
         </is>
       </c>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>PTFE AWG28 전선</t>
+          <t>TBD (두텍 사용품)</t>
         </is>
       </c>
       <c r="I56" s="17" t="inlineStr">
         <is>
-          <t>UL1213 계열 200 °C, 8심 × 60 mm + 수축튜브 (M12 핀 납땜)</t>
+          <t>M12 8핀 수컷 전면 장착형 M16×1.5, 리드선형 (W-2 납땜)</t>
         </is>
       </c>
       <c r="J56" s="19" t="n">
-        <v>0.15</v>
+        <v>2</v>
       </c>
       <c r="K56" s="19" t="n">
-        <v>0.4</v>
+        <v>10</v>
       </c>
       <c r="L56" s="20">
         <f>D56*J56</f>
@@ -4564,9 +4564,9 @@
         <f>D56*K56</f>
         <v/>
       </c>
-      <c r="N56" s="21" t="inlineStr">
-        <is>
-          <t>추정</t>
+      <c r="N56" s="22" t="inlineStr">
+        <is>
+          <t>TBD</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4581,7 @@
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D57" s="18" t="n">
@@ -4604,19 +4604,19 @@
       </c>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>SHR-04V-S</t>
+          <t>GHR-08V-S</t>
         </is>
       </c>
       <c r="I57" s="17" t="inlineStr">
         <is>
-          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
+          <t>GH 1.25 mm 8핀 소켓 하우징 (M12 하네스 W-2)</t>
         </is>
       </c>
       <c r="J57" s="19" t="n">
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
       <c r="K57" s="19" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="L57" s="20">
         <f>D57*J57</f>
@@ -4643,11 +4643,11 @@
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D58" s="18" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
@@ -4666,12 +4666,12 @@
       </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>SSHL-002T-P0.2</t>
         </is>
       </c>
       <c r="I58" s="17" t="inlineStr">
         <is>
-          <t>SH 크림프 단자 AWG 32–28</t>
+          <t>GH 크림프 단자 AWG 30–26</t>
         </is>
       </c>
       <c r="J58" s="19" t="n">
@@ -4705,7 +4705,7 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>W-1</t>
+          <t>W-2</t>
         </is>
       </c>
       <c r="D59" s="18" t="n">
@@ -4728,19 +4728,19 @@
       </c>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>PTFE AWG30 전선</t>
+          <t>PTFE AWG28 전선</t>
         </is>
       </c>
       <c r="I59" s="17" t="inlineStr">
         <is>
-          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
+          <t>UL1213 계열 200 °C, 8심 × 60 mm + 수축튜브 (M12 핀 납땜)</t>
         </is>
       </c>
       <c r="J59" s="19" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="K59" s="19" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="L59" s="20">
         <f>D59*J59</f>
@@ -4762,12 +4762,12 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>조립</t>
+          <t>하네스</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>W-1</t>
         </is>
       </c>
       <c r="D60" s="18" t="n">
@@ -4785,24 +4785,24 @@
       </c>
       <c r="G60" s="16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>SMT 양면 실장</t>
+          <t>SHR-04V-S</t>
         </is>
       </c>
       <c r="I60" s="17" t="inlineStr">
         <is>
-          <t>1k 기준 조립비</t>
+          <t>SH 1.0 mm 4핀 소켓 하우징 (센서 하네스 W-1)</t>
         </is>
       </c>
       <c r="J60" s="19" t="n">
-        <v>2</v>
+        <v>0.04</v>
       </c>
       <c r="K60" s="19" t="n">
-        <v>4</v>
+        <v>0.1</v>
       </c>
       <c r="L60" s="20">
         <f>D60*J60</f>
@@ -4812,24 +4812,210 @@
         <f>D60*K60</f>
         <v/>
       </c>
-      <c r="N60" s="21" t="inlineStr">
+      <c r="N60" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D61" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E61" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G61" s="16" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="H61" s="17" t="inlineStr">
+        <is>
+          <t>SSH-003T-P0.2-H</t>
+        </is>
+      </c>
+      <c r="I61" s="17" t="inlineStr">
+        <is>
+          <t>SH 크림프 단자 AWG 32–28</t>
+        </is>
+      </c>
+      <c r="J61" s="19" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K61" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L61" s="20">
+        <f>D61*J61</f>
+        <v/>
+      </c>
+      <c r="M61" s="20">
+        <f>D61*K61</f>
+        <v/>
+      </c>
+      <c r="N61" s="16" t="inlineStr">
+        <is>
+          <t>제안</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="16" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>하네스</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>W-1</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" s="17" t="inlineStr">
+        <is>
+          <t>PTFE AWG30 전선</t>
+        </is>
+      </c>
+      <c r="I62" s="17" t="inlineStr">
+        <is>
+          <t>UL1213 계열 200 °C, 4심 × 60 mm (HTX99R 뒤 핀 납땜 + 수축튜브)</t>
+        </is>
+      </c>
+      <c r="J62" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K62" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L62" s="20">
+        <f>D62*J62</f>
+        <v/>
+      </c>
+      <c r="M62" s="20">
+        <f>D62*K62</f>
+        <v/>
+      </c>
+      <c r="N62" s="21" t="inlineStr">
         <is>
           <t>추정</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="I61" s="3" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="16" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>조립</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H63" s="17" t="inlineStr">
+        <is>
+          <t>SMT 양면 실장</t>
+        </is>
+      </c>
+      <c r="I63" s="17" t="inlineStr">
+        <is>
+          <t>1k 기준 조립비</t>
+        </is>
+      </c>
+      <c r="J63" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L63" s="20">
+        <f>D63*J63</f>
+        <v/>
+      </c>
+      <c r="M63" s="20">
+        <f>D63*K63</f>
+        <v/>
+      </c>
+      <c r="N63" s="21" t="inlineStr">
+        <is>
+          <t>추정</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="I64" s="3" t="inlineStr">
         <is>
           <t>합계 (1대분)</t>
         </is>
       </c>
-      <c r="L61" s="23">
-        <f>SUM(L2:L60)</f>
-        <v/>
-      </c>
-      <c r="M61" s="23">
-        <f>SUM(M2:M60)</f>
+      <c r="L64" s="23">
+        <f>SUM(L2:L63)</f>
+        <v/>
+      </c>
+      <c r="M64" s="23">
+        <f>SUM(M2:M63)</f>
         <v/>
       </c>
     </row>

</xml_diff>